<commit_message>
[Malterlib/Memory] Reconfigure memory manager to use slab allocator up to < 2 MiB on 4 KiB page platforms (macOS arm64 (16 KiB pages) already was 2 MiB)
</commit_message>
<xml_diff>
--- a/Documentation/MemoryManagerSlabCalculations.xlsx
+++ b/Documentation/MemoryManagerSlabCalculations.xlsx
@@ -1,16 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="24030"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10714"/>
   <workbookPr autoCompressPictures="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/opt/Source/Favro/Malterlib/Memory/Documentation/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20C3338-8FC3-7246-8389-916FB721DF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="60" windowWidth="25600" windowHeight="16060"/>
+    <workbookView xWindow="1620" yWindow="500" windowWidth="45820" windowHeight="28560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="140001" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -54,7 +71,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -172,6 +189,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -463,9 +483,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:AJ485"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A3:AJ515"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="7" width="13.6640625" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
@@ -473,7 +493,7 @@
     <col min="13" max="13" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="L3" t="s">
         <v>6</v>
       </c>
@@ -487,7 +507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G4">
         <v>1</v>
       </c>
@@ -529,7 +549,7 @@
         <v>4095</v>
       </c>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G5">
         <v>2</v>
       </c>
@@ -571,7 +591,7 @@
         <v>4094</v>
       </c>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G6">
         <v>4</v>
       </c>
@@ -617,7 +637,7 @@
         <v>4092</v>
       </c>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G7">
         <v>8</v>
       </c>
@@ -663,7 +683,7 @@
         <v>4088</v>
       </c>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G8">
         <f t="shared" ref="G8:G71" si="8">G7+H8</f>
         <v>12</v>
@@ -709,7 +729,7 @@
         <v>4084</v>
       </c>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G9">
         <f>G8+H9</f>
         <v>16</v>
@@ -756,7 +776,7 @@
         <v>4080</v>
       </c>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G10">
         <f>G9+H10</f>
         <v>20</v>
@@ -803,7 +823,7 @@
         <v>4076</v>
       </c>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G11">
         <f>G10+H11</f>
         <v>24</v>
@@ -850,7 +870,7 @@
         <v>4072</v>
       </c>
     </row>
-    <row r="12" spans="1:19">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G12">
         <f>G11+H12</f>
         <v>28</v>
@@ -897,7 +917,7 @@
         <v>4068</v>
       </c>
     </row>
-    <row r="13" spans="1:19">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G13">
         <f>G12+H13</f>
         <v>32</v>
@@ -944,7 +964,7 @@
         <v>4064</v>
       </c>
     </row>
-    <row r="14" spans="1:19">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -1003,7 +1023,7 @@
         <v>4060</v>
       </c>
     </row>
-    <row r="15" spans="1:19">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" ref="A15:A22" si="12">B15-E15</f>
         <v>3</v>
@@ -1072,7 +1092,7 @@
         <v>4056</v>
       </c>
     </row>
-    <row r="16" spans="1:19">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16">
         <f t="shared" si="12"/>
         <v>1</v>
@@ -1142,7 +1162,7 @@
         <v>4052</v>
       </c>
     </row>
-    <row r="17" spans="1:19">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17">
         <f t="shared" si="12"/>
         <v>1</v>
@@ -1212,7 +1232,7 @@
         <v>4048</v>
       </c>
     </row>
-    <row r="18" spans="1:19">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18">
         <f t="shared" si="12"/>
         <v>4</v>
@@ -1282,7 +1302,7 @@
         <v>4044</v>
       </c>
     </row>
-    <row r="19" spans="1:19">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19">
         <f t="shared" si="12"/>
         <v>1</v>
@@ -1352,7 +1372,7 @@
         <v>4040</v>
       </c>
     </row>
-    <row r="20" spans="1:19">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20">
         <f t="shared" si="12"/>
         <v>1</v>
@@ -1422,7 +1442,7 @@
         <v>4036</v>
       </c>
     </row>
-    <row r="21" spans="1:19">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21">
         <f t="shared" si="12"/>
         <v>1</v>
@@ -1492,7 +1512,7 @@
         <v>4032</v>
       </c>
     </row>
-    <row r="22" spans="1:19">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22">
         <f t="shared" si="12"/>
         <v>1</v>
@@ -1562,7 +1582,7 @@
         <v>4024</v>
       </c>
     </row>
-    <row r="23" spans="1:19">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="E23" t="s">
         <v>2</v>
       </c>
@@ -1617,7 +1637,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="24" spans="1:19">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G24">
         <f t="shared" si="8"/>
         <v>88</v>
@@ -1665,7 +1685,7 @@
         <v>4008</v>
       </c>
     </row>
-    <row r="25" spans="1:19">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G25">
         <f t="shared" si="8"/>
         <v>96</v>
@@ -1713,7 +1733,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="26" spans="1:19">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G26">
         <f t="shared" si="8"/>
         <v>104</v>
@@ -1761,7 +1781,7 @@
         <v>3992</v>
       </c>
     </row>
-    <row r="27" spans="1:19">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G27">
         <f t="shared" si="8"/>
         <v>112</v>
@@ -1809,7 +1829,7 @@
         <v>3984</v>
       </c>
     </row>
-    <row r="28" spans="1:19">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G28">
         <f t="shared" si="8"/>
         <v>120</v>
@@ -1857,7 +1877,7 @@
         <v>3976</v>
       </c>
     </row>
-    <row r="29" spans="1:19">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G29">
         <f t="shared" si="8"/>
         <v>128</v>
@@ -1905,7 +1925,7 @@
         <v>3968</v>
       </c>
     </row>
-    <row r="30" spans="1:19">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G30">
         <f t="shared" si="8"/>
         <v>144</v>
@@ -1952,7 +1972,7 @@
         <v>3952</v>
       </c>
     </row>
-    <row r="31" spans="1:19">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G31">
         <f t="shared" si="8"/>
         <v>160</v>
@@ -2000,7 +2020,7 @@
         <v>3936</v>
       </c>
     </row>
-    <row r="32" spans="1:19">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G32">
         <f t="shared" si="8"/>
         <v>176</v>
@@ -2048,7 +2068,7 @@
         <v>3920</v>
       </c>
     </row>
-    <row r="33" spans="4:19">
+    <row r="33" spans="4:19" x14ac:dyDescent="0.2">
       <c r="G33">
         <f t="shared" si="8"/>
         <v>192</v>
@@ -2096,7 +2116,7 @@
         <v>3904</v>
       </c>
     </row>
-    <row r="34" spans="4:19">
+    <row r="34" spans="4:19" x14ac:dyDescent="0.2">
       <c r="G34">
         <f t="shared" si="8"/>
         <v>208</v>
@@ -2144,7 +2164,7 @@
         <v>3888</v>
       </c>
     </row>
-    <row r="35" spans="4:19">
+    <row r="35" spans="4:19" x14ac:dyDescent="0.2">
       <c r="G35">
         <f t="shared" si="8"/>
         <v>224</v>
@@ -2192,7 +2212,7 @@
         <v>3872</v>
       </c>
     </row>
-    <row r="36" spans="4:19">
+    <row r="36" spans="4:19" x14ac:dyDescent="0.2">
       <c r="G36">
         <f t="shared" si="8"/>
         <v>240</v>
@@ -2240,7 +2260,7 @@
         <v>3856</v>
       </c>
     </row>
-    <row r="37" spans="4:19">
+    <row r="37" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D37">
         <f>I37</f>
         <v>1</v>
@@ -2300,7 +2320,7 @@
         <v>3840</v>
       </c>
     </row>
-    <row r="38" spans="4:19">
+    <row r="38" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D38">
         <f>I38/9</f>
         <v>1</v>
@@ -2359,7 +2379,7 @@
         <v>3808</v>
       </c>
     </row>
-    <row r="39" spans="4:19">
+    <row r="39" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D39">
         <f>I39/5</f>
         <v>1</v>
@@ -2419,7 +2439,7 @@
         <v>3776</v>
       </c>
     </row>
-    <row r="40" spans="4:19">
+    <row r="40" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D40">
         <f>I40/11</f>
         <v>1</v>
@@ -2479,7 +2499,7 @@
         <v>3744</v>
       </c>
     </row>
-    <row r="41" spans="4:19">
+    <row r="41" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D41">
         <f>I41/3</f>
         <v>1</v>
@@ -2539,7 +2559,7 @@
         <v>3712</v>
       </c>
     </row>
-    <row r="42" spans="4:19">
+    <row r="42" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D42">
         <f>I42/13</f>
         <v>1</v>
@@ -2599,7 +2619,7 @@
         <v>3680</v>
       </c>
     </row>
-    <row r="43" spans="4:19">
+    <row r="43" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D43">
         <f>I43/7</f>
         <v>1</v>
@@ -2659,7 +2679,7 @@
         <v>3648</v>
       </c>
     </row>
-    <row r="44" spans="4:19">
+    <row r="44" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D44">
         <f>I44/15</f>
         <v>1</v>
@@ -2719,7 +2739,7 @@
         <v>3616</v>
       </c>
     </row>
-    <row r="45" spans="4:19">
+    <row r="45" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D45">
         <f t="shared" ref="D45" si="21">I45</f>
         <v>1</v>
@@ -2779,7 +2799,7 @@
         <v>3584</v>
       </c>
     </row>
-    <row r="46" spans="4:19">
+    <row r="46" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D46">
         <f t="shared" ref="D46" si="22">I46/9</f>
         <v>1</v>
@@ -2838,7 +2858,7 @@
         <v>3520</v>
       </c>
     </row>
-    <row r="47" spans="4:19">
+    <row r="47" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D47">
         <f t="shared" ref="D47" si="23">I47/5</f>
         <v>1</v>
@@ -2898,7 +2918,7 @@
         <v>3456</v>
       </c>
     </row>
-    <row r="48" spans="4:19">
+    <row r="48" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D48">
         <f t="shared" ref="D48" si="24">I48/11</f>
         <v>1</v>
@@ -2958,7 +2978,7 @@
         <v>3392</v>
       </c>
     </row>
-    <row r="49" spans="4:19">
+    <row r="49" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D49">
         <f t="shared" ref="D49" si="25">I49/3</f>
         <v>1</v>
@@ -3018,7 +3038,7 @@
         <v>3328</v>
       </c>
     </row>
-    <row r="50" spans="4:19">
+    <row r="50" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D50">
         <f t="shared" ref="D50" si="26">I50/13</f>
         <v>1</v>
@@ -3078,7 +3098,7 @@
         <v>3264</v>
       </c>
     </row>
-    <row r="51" spans="4:19">
+    <row r="51" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D51">
         <f t="shared" ref="D51" si="27">I51/7</f>
         <v>1</v>
@@ -3138,7 +3158,7 @@
         <v>3200</v>
       </c>
     </row>
-    <row r="52" spans="4:19">
+    <row r="52" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D52">
         <f t="shared" ref="D52" si="28">I52/15</f>
         <v>1</v>
@@ -3198,7 +3218,7 @@
         <v>3136</v>
       </c>
     </row>
-    <row r="53" spans="4:19">
+    <row r="53" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D53">
         <f t="shared" ref="D53" si="29">I53</f>
         <v>1</v>
@@ -3258,7 +3278,7 @@
         <v>3072</v>
       </c>
     </row>
-    <row r="54" spans="4:19">
+    <row r="54" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D54">
         <f t="shared" ref="D54" si="31">I54/9</f>
         <v>1</v>
@@ -3317,7 +3337,7 @@
         <v>2944</v>
       </c>
     </row>
-    <row r="55" spans="4:19">
+    <row r="55" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D55">
         <f t="shared" ref="D55" si="32">I55/5</f>
         <v>1</v>
@@ -3377,7 +3397,7 @@
         <v>2816</v>
       </c>
     </row>
-    <row r="56" spans="4:19">
+    <row r="56" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D56">
         <f t="shared" ref="D56" si="33">I56/11</f>
         <v>1</v>
@@ -3437,7 +3457,7 @@
         <v>2688</v>
       </c>
     </row>
-    <row r="57" spans="4:19">
+    <row r="57" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D57">
         <f t="shared" ref="D57" si="34">I57/3</f>
         <v>1</v>
@@ -3497,7 +3517,7 @@
         <v>2560</v>
       </c>
     </row>
-    <row r="58" spans="4:19">
+    <row r="58" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D58">
         <f t="shared" ref="D58" si="35">I58/13</f>
         <v>1</v>
@@ -3557,7 +3577,7 @@
         <v>2432</v>
       </c>
     </row>
-    <row r="59" spans="4:19">
+    <row r="59" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D59">
         <f t="shared" ref="D59" si="36">I59/7</f>
         <v>1</v>
@@ -3617,7 +3637,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="60" spans="4:19">
+    <row r="60" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D60">
         <f t="shared" ref="D60" si="37">I60/15</f>
         <v>1</v>
@@ -3677,7 +3697,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="61" spans="4:19">
+    <row r="61" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D61">
         <f t="shared" ref="D61" si="38">I61</f>
         <v>1</v>
@@ -3737,7 +3757,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="62" spans="4:19">
+    <row r="62" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D62">
         <f t="shared" ref="D62" si="40">I62/9</f>
         <v>1</v>
@@ -3796,7 +3816,7 @@
         <v>1792</v>
       </c>
     </row>
-    <row r="63" spans="4:19">
+    <row r="63" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D63">
         <f t="shared" ref="D63" si="41">I63/5</f>
         <v>1</v>
@@ -3856,7 +3876,7 @@
         <v>1536</v>
       </c>
     </row>
-    <row r="64" spans="4:19">
+    <row r="64" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D64">
         <f t="shared" ref="D64" si="42">I64/11</f>
         <v>1</v>
@@ -3916,7 +3936,7 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="65" spans="4:19">
+    <row r="65" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D65">
         <f t="shared" ref="D65" si="43">I65/3</f>
         <v>1</v>
@@ -3976,7 +3996,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="66" spans="4:19">
+    <row r="66" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D66">
         <f t="shared" ref="D66" si="44">I66/13</f>
         <v>1</v>
@@ -4036,7 +4056,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="67" spans="4:19">
+    <row r="67" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D67">
         <f t="shared" ref="D67" si="45">I67/7</f>
         <v>1</v>
@@ -4096,7 +4116,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="68" spans="4:19">
+    <row r="68" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D68">
         <f t="shared" ref="D68" si="47">I68/15</f>
         <v>1</v>
@@ -4156,7 +4176,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="69" spans="4:19">
+    <row r="69" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D69">
         <f t="shared" ref="D69" si="49">I69</f>
         <v>1</v>
@@ -4216,7 +4236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="4:19">
+    <row r="70" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D70">
         <f t="shared" ref="D70" si="52">I70/9</f>
         <v>1</v>
@@ -4275,7 +4295,7 @@
         <v>3584</v>
       </c>
     </row>
-    <row r="71" spans="4:19">
+    <row r="71" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D71">
         <f t="shared" ref="D71" si="53">I71/5</f>
         <v>1</v>
@@ -4335,7 +4355,7 @@
         <v>3072</v>
       </c>
     </row>
-    <row r="72" spans="4:19">
+    <row r="72" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D72">
         <f t="shared" ref="D72" si="55">I72/11</f>
         <v>1</v>
@@ -4395,7 +4415,7 @@
         <v>2560</v>
       </c>
     </row>
-    <row r="73" spans="4:19">
+    <row r="73" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D73">
         <f t="shared" ref="D73" si="59">I73/3</f>
         <v>1</v>
@@ -4455,7 +4475,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="74" spans="4:19">
+    <row r="74" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D74">
         <f t="shared" ref="D74" si="62">I74/13</f>
         <v>1</v>
@@ -4515,7 +4535,7 @@
         <v>1536</v>
       </c>
     </row>
-    <row r="75" spans="4:19">
+    <row r="75" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D75">
         <f t="shared" ref="D75" si="63">I75/7</f>
         <v>1</v>
@@ -4575,7 +4595,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="76" spans="4:19">
+    <row r="76" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D76">
         <f t="shared" ref="D76" si="64">I76/15</f>
         <v>1</v>
@@ -4635,7 +4655,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="77" spans="4:19">
+    <row r="77" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D77">
         <f t="shared" ref="D77" si="65">I77</f>
         <v>2</v>
@@ -4695,7 +4715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="4:19">
+    <row r="78" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D78">
         <f t="shared" ref="D78" si="67">I78/9</f>
         <v>1</v>
@@ -4754,7 +4774,7 @@
         <v>3072</v>
       </c>
     </row>
-    <row r="79" spans="4:19">
+    <row r="79" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D79">
         <f t="shared" ref="D79" si="68">I79/5</f>
         <v>1</v>
@@ -4814,7 +4834,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="80" spans="4:19">
+    <row r="80" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D80">
         <f t="shared" ref="D80" si="69">I80/11</f>
         <v>1</v>
@@ -4874,7 +4894,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="81" spans="4:19">
+    <row r="81" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D81">
         <f t="shared" ref="D81" si="70">I81/3</f>
         <v>1</v>
@@ -4934,7 +4954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="4:19">
+    <row r="82" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D82">
         <f t="shared" ref="D82" si="71">I82/13</f>
         <v>1</v>
@@ -4994,7 +5014,7 @@
         <v>3072</v>
       </c>
     </row>
-    <row r="83" spans="4:19">
+    <row r="83" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D83">
         <f t="shared" ref="D83" si="72">I83/7</f>
         <v>1</v>
@@ -5054,7 +5074,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="84" spans="4:19">
+    <row r="84" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D84">
         <f t="shared" ref="D84" si="73">I84/15</f>
         <v>1</v>
@@ -5114,7 +5134,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="85" spans="4:19">
+    <row r="85" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D85">
         <f t="shared" ref="D85" si="74">I85</f>
         <v>4</v>
@@ -5174,7 +5194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="4:19">
+    <row r="86" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D86">
         <f t="shared" ref="D86" si="76">I86/9</f>
         <v>1</v>
@@ -5233,7 +5253,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="87" spans="4:19">
+    <row r="87" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D87">
         <f t="shared" ref="D87" si="77">I87/5</f>
         <v>1</v>
@@ -5293,7 +5313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="4:19">
+    <row r="88" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D88">
         <f t="shared" ref="D88" si="78">I88/11</f>
         <v>1</v>
@@ -5353,7 +5373,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="89" spans="4:19">
+    <row r="89" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D89">
         <f t="shared" ref="D89" si="80">I89/3</f>
         <v>2</v>
@@ -5413,7 +5433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="4:19">
+    <row r="90" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D90">
         <f t="shared" ref="D90" si="82">I90/13</f>
         <v>1</v>
@@ -5473,7 +5493,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="91" spans="4:19">
+    <row r="91" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D91">
         <f t="shared" ref="D91" si="83">I91/7</f>
         <v>1</v>
@@ -5533,7 +5553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="4:19">
+    <row r="92" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D92">
         <f t="shared" ref="D92" si="84">I92/15</f>
         <v>1</v>
@@ -5593,7 +5613,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="93" spans="4:19">
+    <row r="93" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D93">
         <f t="shared" ref="D93" si="85">I93</f>
         <v>8</v>
@@ -5653,7 +5673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="4:19">
+    <row r="94" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D94">
         <f t="shared" ref="D94" si="87">I94/9</f>
         <v>1</v>
@@ -5712,7 +5732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="4:19">
+    <row r="95" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D95">
         <f t="shared" ref="D95" si="94">I95/5</f>
         <v>2</v>
@@ -5730,7 +5750,7 @@
         <v>40960</v>
       </c>
       <c r="H95">
-        <f t="shared" ref="H95:H157" si="95">H94</f>
+        <f t="shared" ref="H95:H140" si="95">H94</f>
         <v>4096</v>
       </c>
       <c r="I95">
@@ -5772,7 +5792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="4:19">
+    <row r="96" spans="4:19" x14ac:dyDescent="0.2">
       <c r="D96">
         <f t="shared" ref="D96" si="96">I96/11</f>
         <v>1</v>
@@ -5832,7 +5852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="4:30">
+    <row r="97" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D97">
         <f t="shared" ref="D97" si="97">I97/3</f>
         <v>4</v>
@@ -5892,7 +5912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="4:30">
+    <row r="98" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D98">
         <f t="shared" ref="D98" si="98">I98/13</f>
         <v>1</v>
@@ -5952,7 +5972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="4:30">
+    <row r="99" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D99">
         <f t="shared" ref="D99" si="99">I99/7</f>
         <v>2</v>
@@ -6012,7 +6032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="4:30">
+    <row r="100" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D100">
         <f t="shared" ref="D100" si="101">I100/15</f>
         <v>1</v>
@@ -6072,7 +6092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="4:30">
+    <row r="101" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D101">
         <f t="shared" ref="D101" si="102">I101</f>
         <v>16</v>
@@ -6133,7 +6153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="4:30">
+    <row r="102" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D102">
         <f t="shared" ref="D102" si="105">I102/9</f>
         <v>2</v>
@@ -6177,7 +6197,7 @@
         <v>18</v>
       </c>
       <c r="O102">
-        <f t="shared" ref="O102:O165" si="111">O94*2</f>
+        <f t="shared" ref="O102:O140" si="111">O94*2</f>
         <v>4096</v>
       </c>
       <c r="P102">
@@ -6193,7 +6213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="4:30">
+    <row r="103" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D103">
         <f t="shared" ref="D103" si="113">I103/5</f>
         <v>4</v>
@@ -6254,7 +6274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="4:30">
+    <row r="104" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D104">
         <f t="shared" ref="D104" si="115">I104/11</f>
         <v>2</v>
@@ -6315,7 +6335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="4:30">
+    <row r="105" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D105">
         <f t="shared" ref="D105" si="116">I105/3</f>
         <v>8</v>
@@ -6376,7 +6396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="4:30">
+    <row r="106" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D106">
         <f t="shared" ref="D106" si="117">I106/13</f>
         <v>2</v>
@@ -6437,7 +6457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="4:30">
+    <row r="107" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D107">
         <f t="shared" ref="D107" si="118">I107/7</f>
         <v>4</v>
@@ -6498,7 +6518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="4:30">
+    <row r="108" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D108">
         <f t="shared" ref="D108" si="119">I108/15</f>
         <v>2</v>
@@ -6559,7 +6579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="4:30">
+    <row r="109" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D109">
         <f t="shared" ref="D109" si="120">I109</f>
         <v>32</v>
@@ -6620,7 +6640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="4:30">
+    <row r="110" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D110">
         <f t="shared" ref="D110" si="122">I110/9</f>
         <v>4</v>
@@ -6682,7 +6702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="4:30">
+    <row r="111" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D111">
         <f t="shared" ref="D111" si="129">I111/5</f>
         <v>8</v>
@@ -6704,7 +6724,7 @@
         <v>16384</v>
       </c>
       <c r="I111">
-        <f t="shared" ref="I111:I174" si="130">I103*2</f>
+        <f t="shared" ref="I111:I140" si="130">I103*2</f>
         <v>40</v>
       </c>
       <c r="J111">
@@ -6744,7 +6764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="4:30">
+    <row r="112" spans="4:30" x14ac:dyDescent="0.2">
       <c r="D112">
         <f t="shared" ref="D112" si="131">I112/11</f>
         <v>4</v>
@@ -6808,7 +6828,7 @@
       <c r="AC112" s="1"/>
       <c r="AD112" s="1"/>
     </row>
-    <row r="113" spans="3:36">
+    <row r="113" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D113">
         <f t="shared" ref="D113" si="132">I113/3</f>
         <v>16</v>
@@ -6876,7 +6896,7 @@
       <c r="AC113" s="1"/>
       <c r="AD113" s="1"/>
     </row>
-    <row r="114" spans="3:36">
+    <row r="114" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D114">
         <f t="shared" ref="D114" si="133">I114/13</f>
         <v>4</v>
@@ -6956,7 +6976,7 @@
         <v>254205</v>
       </c>
     </row>
-    <row r="115" spans="3:36">
+    <row r="115" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D115">
         <f t="shared" ref="D115" si="134">I115/7</f>
         <v>8</v>
@@ -7028,7 +7048,7 @@
         <v>62.061767578125</v>
       </c>
     </row>
-    <row r="116" spans="3:36">
+    <row r="116" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D116">
         <f t="shared" ref="D116" si="135">I116/15</f>
         <v>4</v>
@@ -7096,7 +7116,7 @@
       <c r="AC116" s="1"/>
       <c r="AD116" s="1"/>
     </row>
-    <row r="117" spans="3:36">
+    <row r="117" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D117">
         <f t="shared" ref="D117" si="136">I117</f>
         <v>64</v>
@@ -7160,7 +7180,7 @@
       <c r="AC117" s="1"/>
       <c r="AD117" s="1"/>
     </row>
-    <row r="118" spans="3:36">
+    <row r="118" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D118">
         <f t="shared" ref="D118" si="138">I118/9</f>
         <v>8</v>
@@ -7174,7 +7194,7 @@
         <v>56.875</v>
       </c>
       <c r="G118">
-        <f t="shared" ref="G118:G181" si="139">G117+H118</f>
+        <f t="shared" ref="G118:G125" si="139">G117+H118</f>
         <v>294912</v>
       </c>
       <c r="H118">
@@ -7190,19 +7210,19 @@
         <v>294912</v>
       </c>
       <c r="K118">
-        <f t="shared" ref="K118:K124" si="140">FLOOR(J118/G118,1)</f>
+        <f t="shared" ref="K118:K125" si="140">FLOOR(J118/G118,1)</f>
         <v>1</v>
       </c>
       <c r="L118" s="1">
-        <f t="shared" ref="L118:L124" si="141">(J118-K118*G118)/J118</f>
+        <f t="shared" ref="L118:L125" si="141">(J118-K118*G118)/J118</f>
         <v>0</v>
       </c>
       <c r="M118" s="1">
-        <f t="shared" ref="M118:M124" si="142">(G118-(G117+1))/(G118)</f>
+        <f t="shared" ref="M118:M125" si="142">(G118-(G117+1))/(G118)</f>
         <v>0.11110772026909722</v>
       </c>
       <c r="N118">
-        <f t="shared" ref="N118:N124" si="143">J118/4096</f>
+        <f t="shared" ref="N118:N125" si="143">J118/4096</f>
         <v>72</v>
       </c>
       <c r="O118">
@@ -7214,7 +7234,7 @@
         <v>0</v>
       </c>
       <c r="Q118">
-        <f t="shared" ref="Q118:Q124" si="144">P118/I118</f>
+        <f t="shared" ref="Q118:Q125" si="144">P118/I118</f>
         <v>0</v>
       </c>
       <c r="S118">
@@ -7224,7 +7244,7 @@
       <c r="AC118" s="1"/>
       <c r="AD118" s="1"/>
     </row>
-    <row r="119" spans="3:36">
+    <row r="119" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D119">
         <f t="shared" ref="D119" si="145">I119/5</f>
         <v>16</v>
@@ -7288,7 +7308,7 @@
       <c r="AC119" s="1"/>
       <c r="AD119" s="1"/>
     </row>
-    <row r="120" spans="3:36">
+    <row r="120" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D120">
         <f t="shared" ref="D120" si="146">I120/11</f>
         <v>8</v>
@@ -7352,7 +7372,7 @@
       <c r="AC120" s="1"/>
       <c r="AD120" s="1"/>
     </row>
-    <row r="121" spans="3:36">
+    <row r="121" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D121">
         <f t="shared" ref="D121" si="147">I121/3</f>
         <v>32</v>
@@ -7416,7 +7436,7 @@
       <c r="AC121" s="1"/>
       <c r="AD121" s="1"/>
     </row>
-    <row r="122" spans="3:36">
+    <row r="122" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D122">
         <f t="shared" ref="D122" si="148">I122/13</f>
         <v>8</v>
@@ -7480,7 +7500,7 @@
       <c r="AC122" s="1"/>
       <c r="AD122" s="1"/>
     </row>
-    <row r="123" spans="3:36">
+    <row r="123" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D123">
         <f t="shared" ref="D123" si="149">I123/7</f>
         <v>16</v>
@@ -7544,7 +7564,7 @@
       <c r="AC123" s="1"/>
       <c r="AD123" s="1"/>
     </row>
-    <row r="124" spans="3:36">
+    <row r="124" spans="4:36" x14ac:dyDescent="0.2">
       <c r="D124">
         <f t="shared" ref="D124" si="150">I124/15</f>
         <v>8</v>
@@ -7554,7 +7574,7 @@
         <v>3.663003663003663E-3</v>
       </c>
       <c r="F124">
-        <f t="shared" ref="F124:F187" si="151">$E$22/I124</f>
+        <f t="shared" ref="F124" si="151">$E$22/I124</f>
         <v>34.125</v>
       </c>
       <c r="G124">
@@ -7608,1822 +7628,2944 @@
       <c r="AC124" s="1"/>
       <c r="AD124" s="1"/>
     </row>
-    <row r="125" spans="3:36">
-      <c r="E125" s="1"/>
-      <c r="L125" s="1"/>
-      <c r="M125" s="1"/>
-    </row>
-    <row r="126" spans="3:36">
-      <c r="C126" t="s">
-        <v>8</v>
-      </c>
-      <c r="E126" s="1"/>
-      <c r="L126" s="1"/>
+    <row r="125" spans="4:36" x14ac:dyDescent="0.2">
+      <c r="D125">
+        <f t="shared" ref="D125:D133" si="152">I125</f>
+        <v>128</v>
+      </c>
+      <c r="E125" s="1">
+        <f t="shared" ref="E125:E133" si="153">(F125 - FLOOR(F125,1))/F125</f>
+        <v>3.05399462496946E-2</v>
+      </c>
+      <c r="F125">
+        <f t="shared" ref="F125:F133" si="154">$E$15/I125</f>
+        <v>31.9765625</v>
+      </c>
+      <c r="G125">
+        <f t="shared" si="139"/>
+        <v>524288</v>
+      </c>
+      <c r="H125">
+        <f t="shared" si="95"/>
+        <v>32768</v>
+      </c>
+      <c r="I125">
+        <f t="shared" si="130"/>
+        <v>128</v>
+      </c>
+      <c r="J125">
+        <f t="shared" ref="J125:J133" si="155">4096*I125</f>
+        <v>524288</v>
+      </c>
+      <c r="K125">
+        <f t="shared" si="140"/>
+        <v>1</v>
+      </c>
+      <c r="L125" s="1">
+        <f t="shared" si="141"/>
+        <v>0</v>
+      </c>
+      <c r="M125" s="1">
+        <f t="shared" si="142"/>
+        <v>6.2498092651367188E-2</v>
+      </c>
+      <c r="N125">
+        <f t="shared" si="143"/>
+        <v>128</v>
+      </c>
+      <c r="O125">
+        <f t="shared" si="111"/>
+        <v>524288</v>
+      </c>
+      <c r="P125">
+        <f t="shared" ref="P125:P133" si="156">J125-G125*K125</f>
+        <v>0</v>
+      </c>
+      <c r="Q125">
+        <f t="shared" si="144"/>
+        <v>0</v>
+      </c>
+      <c r="S125">
+        <f t="shared" ref="S125:S133" si="157">FLOOR((G125 + 4095)/4096, 1)*4096 - G125</f>
+        <v>0</v>
+      </c>
+      <c r="AC125" s="1"/>
+      <c r="AD125" s="1"/>
+    </row>
+    <row r="126" spans="4:36" x14ac:dyDescent="0.2">
+      <c r="D126">
+        <f t="shared" ref="D126:D133" si="158">I126/9</f>
+        <v>16</v>
+      </c>
+      <c r="E126" s="1">
+        <f t="shared" si="153"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="F126">
+        <f t="shared" ref="F126:F133" si="159">$E$16/I126</f>
+        <v>28.4375</v>
+      </c>
+      <c r="G126">
+        <f t="shared" ref="G126:G133" si="160">G125+H126</f>
+        <v>589824</v>
+      </c>
+      <c r="H126">
+        <f t="shared" ref="H126" si="161">H118*2</f>
+        <v>65536</v>
+      </c>
+      <c r="I126">
+        <f t="shared" si="130"/>
+        <v>144</v>
+      </c>
+      <c r="J126">
+        <f t="shared" si="155"/>
+        <v>589824</v>
+      </c>
+      <c r="K126">
+        <f t="shared" ref="K126:K133" si="162">FLOOR(J126/G126,1)</f>
+        <v>1</v>
+      </c>
+      <c r="L126" s="1">
+        <f t="shared" ref="L126:L133" si="163">(J126-K126*G126)/J126</f>
+        <v>0</v>
+      </c>
       <c r="M126" s="1">
-        <f>MAX(M13:M124)</f>
-        <v>0.11110772026909722</v>
-      </c>
-    </row>
-    <row r="127" spans="3:36">
-      <c r="C127" t="s">
-        <v>9</v>
-      </c>
-      <c r="E127" s="1"/>
-      <c r="L127" s="1"/>
+        <f t="shared" ref="M126:M133" si="164">(G126-(G125+1))/(G126)</f>
+        <v>0.11110941569010417</v>
+      </c>
+      <c r="N126">
+        <f t="shared" ref="N126:N133" si="165">J126/4096</f>
+        <v>144</v>
+      </c>
+      <c r="O126">
+        <f t="shared" si="111"/>
+        <v>32768</v>
+      </c>
+      <c r="P126">
+        <f t="shared" si="156"/>
+        <v>0</v>
+      </c>
+      <c r="Q126">
+        <f t="shared" ref="Q126:Q133" si="166">P126/I126</f>
+        <v>0</v>
+      </c>
+      <c r="S126">
+        <f t="shared" si="157"/>
+        <v>0</v>
+      </c>
+      <c r="AC126" s="1"/>
+      <c r="AD126" s="1"/>
+    </row>
+    <row r="127" spans="4:36" x14ac:dyDescent="0.2">
+      <c r="D127">
+        <f t="shared" ref="D127:D133" si="167">I127/5</f>
+        <v>32</v>
+      </c>
+      <c r="E127" s="1">
+        <f t="shared" si="153"/>
+        <v>2.31990231990232E-2</v>
+      </c>
+      <c r="F127">
+        <f t="shared" ref="F127:F133" si="168">$E$17/I127</f>
+        <v>25.59375</v>
+      </c>
+      <c r="G127">
+        <f t="shared" si="160"/>
+        <v>655360</v>
+      </c>
+      <c r="H127">
+        <f t="shared" si="95"/>
+        <v>65536</v>
+      </c>
+      <c r="I127">
+        <f t="shared" si="130"/>
+        <v>160</v>
+      </c>
+      <c r="J127">
+        <f t="shared" si="155"/>
+        <v>655360</v>
+      </c>
+      <c r="K127">
+        <f t="shared" si="162"/>
+        <v>1</v>
+      </c>
+      <c r="L127" s="1">
+        <f t="shared" si="163"/>
+        <v>0</v>
+      </c>
       <c r="M127" s="1">
-        <f>AVERAGE(M13:M124)</f>
-        <v>8.017894746975085E-2</v>
-      </c>
-    </row>
-    <row r="128" spans="3:36">
-      <c r="E128" s="1"/>
-      <c r="L128" s="1"/>
-      <c r="M128" s="1"/>
-    </row>
-    <row r="129" spans="5:13">
-      <c r="E129" s="1"/>
-      <c r="L129" s="1"/>
-      <c r="M129" s="1"/>
-    </row>
-    <row r="130" spans="5:13">
-      <c r="E130" s="1"/>
-      <c r="L130" s="1"/>
-      <c r="M130" s="1"/>
-    </row>
-    <row r="131" spans="5:13">
-      <c r="E131" s="1"/>
-      <c r="L131" s="1"/>
-      <c r="M131" s="1"/>
-    </row>
-    <row r="132" spans="5:13">
-      <c r="E132" s="1"/>
-      <c r="L132" s="1"/>
-      <c r="M132" s="1"/>
-    </row>
-    <row r="133" spans="5:13">
-      <c r="E133" s="1"/>
-      <c r="L133" s="1"/>
-      <c r="M133" s="1"/>
-    </row>
-    <row r="134" spans="5:13">
-      <c r="E134" s="1"/>
-      <c r="L134" s="1"/>
-      <c r="M134" s="1"/>
-    </row>
-    <row r="135" spans="5:13">
-      <c r="E135" s="1"/>
-      <c r="L135" s="1"/>
-      <c r="M135" s="1"/>
-    </row>
-    <row r="136" spans="5:13">
-      <c r="E136" s="1"/>
-      <c r="L136" s="1"/>
-      <c r="M136" s="1"/>
-    </row>
-    <row r="137" spans="5:13">
-      <c r="E137" s="1"/>
-      <c r="L137" s="1"/>
-      <c r="M137" s="1"/>
-    </row>
-    <row r="138" spans="5:13">
-      <c r="E138" s="1"/>
-      <c r="L138" s="1"/>
-      <c r="M138" s="1"/>
-    </row>
-    <row r="139" spans="5:13">
-      <c r="E139" s="1"/>
-      <c r="L139" s="1"/>
-      <c r="M139" s="1"/>
-    </row>
-    <row r="140" spans="5:13">
-      <c r="E140" s="1"/>
-      <c r="L140" s="1"/>
-      <c r="M140" s="1"/>
-    </row>
-    <row r="141" spans="5:13">
+        <f t="shared" si="164"/>
+        <v>9.999847412109375E-2</v>
+      </c>
+      <c r="N127">
+        <f t="shared" si="165"/>
+        <v>160</v>
+      </c>
+      <c r="O127">
+        <f t="shared" si="111"/>
+        <v>65536</v>
+      </c>
+      <c r="P127">
+        <f t="shared" si="156"/>
+        <v>0</v>
+      </c>
+      <c r="Q127">
+        <f t="shared" si="166"/>
+        <v>0</v>
+      </c>
+      <c r="S127">
+        <f t="shared" si="157"/>
+        <v>0</v>
+      </c>
+      <c r="AC127" s="1"/>
+      <c r="AD127" s="1"/>
+    </row>
+    <row r="128" spans="4:36" x14ac:dyDescent="0.2">
+      <c r="D128">
+        <f t="shared" ref="D128:D133" si="169">I128/11</f>
+        <v>16</v>
+      </c>
+      <c r="E128" s="1">
+        <f t="shared" si="153"/>
+        <v>1.0752688172043012E-2</v>
+      </c>
+      <c r="F128">
+        <f t="shared" ref="F128:F133" si="170">$E$18/I128</f>
+        <v>23.25</v>
+      </c>
+      <c r="G128">
+        <f t="shared" si="160"/>
+        <v>720896</v>
+      </c>
+      <c r="H128">
+        <f t="shared" si="95"/>
+        <v>65536</v>
+      </c>
+      <c r="I128">
+        <f t="shared" si="130"/>
+        <v>176</v>
+      </c>
+      <c r="J128">
+        <f t="shared" si="155"/>
+        <v>720896</v>
+      </c>
+      <c r="K128">
+        <f t="shared" si="162"/>
+        <v>1</v>
+      </c>
+      <c r="L128" s="1">
+        <f t="shared" si="163"/>
+        <v>0</v>
+      </c>
+      <c r="M128" s="1">
+        <f t="shared" si="164"/>
+        <v>9.0907703746448867E-2</v>
+      </c>
+      <c r="N128">
+        <f t="shared" si="165"/>
+        <v>176</v>
+      </c>
+      <c r="O128">
+        <f t="shared" si="111"/>
+        <v>32768</v>
+      </c>
+      <c r="P128">
+        <f t="shared" si="156"/>
+        <v>0</v>
+      </c>
+      <c r="Q128">
+        <f t="shared" si="166"/>
+        <v>0</v>
+      </c>
+      <c r="S128">
+        <f t="shared" si="157"/>
+        <v>0</v>
+      </c>
+      <c r="AC128" s="1"/>
+      <c r="AD128" s="1"/>
+    </row>
+    <row r="129" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D129">
+        <f t="shared" ref="D129:D133" si="171">I129/3</f>
+        <v>64</v>
+      </c>
+      <c r="E129" s="1">
+        <f t="shared" si="153"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="F129">
+        <f t="shared" ref="F129:F133" si="172">$E$19/I129</f>
+        <v>21.328125</v>
+      </c>
+      <c r="G129">
+        <f t="shared" si="160"/>
+        <v>786432</v>
+      </c>
+      <c r="H129">
+        <f t="shared" si="95"/>
+        <v>65536</v>
+      </c>
+      <c r="I129">
+        <f t="shared" si="130"/>
+        <v>192</v>
+      </c>
+      <c r="J129">
+        <f t="shared" si="155"/>
+        <v>786432</v>
+      </c>
+      <c r="K129">
+        <f t="shared" si="162"/>
+        <v>1</v>
+      </c>
+      <c r="L129" s="1">
+        <f t="shared" si="163"/>
+        <v>0</v>
+      </c>
+      <c r="M129" s="1">
+        <f t="shared" si="164"/>
+        <v>8.3332061767578125E-2</v>
+      </c>
+      <c r="N129">
+        <f t="shared" si="165"/>
+        <v>192</v>
+      </c>
+      <c r="O129">
+        <f t="shared" si="111"/>
+        <v>131072</v>
+      </c>
+      <c r="P129">
+        <f t="shared" si="156"/>
+        <v>0</v>
+      </c>
+      <c r="Q129">
+        <f t="shared" si="166"/>
+        <v>0</v>
+      </c>
+      <c r="S129">
+        <f t="shared" si="157"/>
+        <v>0</v>
+      </c>
+      <c r="AC129" s="1"/>
+      <c r="AD129" s="1"/>
+    </row>
+    <row r="130" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D130">
+        <f t="shared" ref="D130:D133" si="173">I130/13</f>
+        <v>16</v>
+      </c>
+      <c r="E130" s="1">
+        <f t="shared" si="153"/>
+        <v>3.4920634920634921E-2</v>
+      </c>
+      <c r="F130">
+        <f t="shared" ref="F130:F133" si="174">$E$20/I130</f>
+        <v>19.6875</v>
+      </c>
+      <c r="G130">
+        <f t="shared" si="160"/>
+        <v>851968</v>
+      </c>
+      <c r="H130">
+        <f t="shared" si="95"/>
+        <v>65536</v>
+      </c>
+      <c r="I130">
+        <f t="shared" si="130"/>
+        <v>208</v>
+      </c>
+      <c r="J130">
+        <f t="shared" si="155"/>
+        <v>851968</v>
+      </c>
+      <c r="K130">
+        <f t="shared" si="162"/>
+        <v>1</v>
+      </c>
+      <c r="L130" s="1">
+        <f t="shared" si="163"/>
+        <v>0</v>
+      </c>
+      <c r="M130" s="1">
+        <f t="shared" si="164"/>
+        <v>7.6921903170072109E-2</v>
+      </c>
+      <c r="N130">
+        <f t="shared" si="165"/>
+        <v>208</v>
+      </c>
+      <c r="O130">
+        <f t="shared" si="111"/>
+        <v>32768</v>
+      </c>
+      <c r="P130">
+        <f t="shared" si="156"/>
+        <v>0</v>
+      </c>
+      <c r="Q130">
+        <f t="shared" si="166"/>
+        <v>0</v>
+      </c>
+      <c r="S130">
+        <f t="shared" si="157"/>
+        <v>0</v>
+      </c>
+      <c r="AC130" s="1"/>
+      <c r="AD130" s="1"/>
+    </row>
+    <row r="131" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D131">
+        <f t="shared" ref="D131:D133" si="175">I131/7</f>
+        <v>32</v>
+      </c>
+      <c r="E131" s="1">
+        <f t="shared" si="153"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="F131">
+        <f t="shared" ref="F131:F133" si="176">$E$21/I131</f>
+        <v>18.28125</v>
+      </c>
+      <c r="G131">
+        <f t="shared" si="160"/>
+        <v>917504</v>
+      </c>
+      <c r="H131">
+        <f t="shared" si="95"/>
+        <v>65536</v>
+      </c>
+      <c r="I131">
+        <f t="shared" si="130"/>
+        <v>224</v>
+      </c>
+      <c r="J131">
+        <f t="shared" si="155"/>
+        <v>917504</v>
+      </c>
+      <c r="K131">
+        <f t="shared" si="162"/>
+        <v>1</v>
+      </c>
+      <c r="L131" s="1">
+        <f t="shared" si="163"/>
+        <v>0</v>
+      </c>
+      <c r="M131" s="1">
+        <f t="shared" si="164"/>
+        <v>7.1427481515066962E-2</v>
+      </c>
+      <c r="N131">
+        <f t="shared" si="165"/>
+        <v>224</v>
+      </c>
+      <c r="O131">
+        <f t="shared" si="111"/>
+        <v>65536</v>
+      </c>
+      <c r="P131">
+        <f t="shared" si="156"/>
+        <v>0</v>
+      </c>
+      <c r="Q131">
+        <f t="shared" si="166"/>
+        <v>0</v>
+      </c>
+      <c r="S131">
+        <f t="shared" si="157"/>
+        <v>0</v>
+      </c>
+      <c r="AC131" s="1"/>
+      <c r="AD131" s="1"/>
+    </row>
+    <row r="132" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D132">
+        <f t="shared" ref="D132:D133" si="177">I132/15</f>
+        <v>16</v>
+      </c>
+      <c r="E132" s="1">
+        <f t="shared" si="153"/>
+        <v>3.663003663003663E-3</v>
+      </c>
+      <c r="F132">
+        <f t="shared" ref="F132:F133" si="178">$E$22/I132</f>
+        <v>17.0625</v>
+      </c>
+      <c r="G132">
+        <f t="shared" si="160"/>
+        <v>983040</v>
+      </c>
+      <c r="H132">
+        <f t="shared" si="95"/>
+        <v>65536</v>
+      </c>
+      <c r="I132">
+        <f t="shared" si="130"/>
+        <v>240</v>
+      </c>
+      <c r="J132">
+        <f t="shared" si="155"/>
+        <v>983040</v>
+      </c>
+      <c r="K132">
+        <f t="shared" si="162"/>
+        <v>1</v>
+      </c>
+      <c r="L132" s="1">
+        <f t="shared" si="163"/>
+        <v>0</v>
+      </c>
+      <c r="M132" s="1">
+        <f t="shared" si="164"/>
+        <v>6.66656494140625E-2</v>
+      </c>
+      <c r="N132">
+        <f t="shared" si="165"/>
+        <v>240</v>
+      </c>
+      <c r="O132">
+        <f t="shared" si="111"/>
+        <v>32768</v>
+      </c>
+      <c r="P132">
+        <f t="shared" si="156"/>
+        <v>0</v>
+      </c>
+      <c r="Q132">
+        <f t="shared" si="166"/>
+        <v>0</v>
+      </c>
+      <c r="S132">
+        <f t="shared" si="157"/>
+        <v>0</v>
+      </c>
+      <c r="AC132" s="1"/>
+      <c r="AD132" s="1"/>
+    </row>
+    <row r="133" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D133">
+        <f t="shared" ref="D133:D140" si="179">I133</f>
+        <v>256</v>
+      </c>
+      <c r="E133" s="1">
+        <f t="shared" ref="E133:E140" si="180">(F133 - FLOOR(F133,1))/F133</f>
+        <v>6.1812851209381875E-2</v>
+      </c>
+      <c r="F133">
+        <f t="shared" ref="F133:F140" si="181">$E$15/I133</f>
+        <v>15.98828125</v>
+      </c>
+      <c r="G133">
+        <f t="shared" si="160"/>
+        <v>1048576</v>
+      </c>
+      <c r="H133">
+        <f t="shared" si="95"/>
+        <v>65536</v>
+      </c>
+      <c r="I133">
+        <f t="shared" si="130"/>
+        <v>256</v>
+      </c>
+      <c r="J133">
+        <f t="shared" ref="J133:J140" si="182">4096*I133</f>
+        <v>1048576</v>
+      </c>
+      <c r="K133">
+        <f t="shared" si="162"/>
+        <v>1</v>
+      </c>
+      <c r="L133" s="1">
+        <f t="shared" si="163"/>
+        <v>0</v>
+      </c>
+      <c r="M133" s="1">
+        <f t="shared" si="164"/>
+        <v>6.2499046325683594E-2</v>
+      </c>
+      <c r="N133">
+        <f t="shared" si="165"/>
+        <v>256</v>
+      </c>
+      <c r="O133">
+        <f t="shared" si="111"/>
+        <v>1048576</v>
+      </c>
+      <c r="P133">
+        <f t="shared" ref="P133:P140" si="183">J133-G133*K133</f>
+        <v>0</v>
+      </c>
+      <c r="Q133">
+        <f t="shared" si="166"/>
+        <v>0</v>
+      </c>
+      <c r="S133">
+        <f t="shared" ref="S133:S140" si="184">FLOOR((G133 + 4095)/4096, 1)*4096 - G133</f>
+        <v>0</v>
+      </c>
+      <c r="AC133" s="1"/>
+      <c r="AD133" s="1"/>
+    </row>
+    <row r="134" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D134">
+        <f t="shared" ref="D134:D140" si="185">I134/9</f>
+        <v>32</v>
+      </c>
+      <c r="E134" s="1">
+        <f t="shared" si="180"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="F134">
+        <f t="shared" ref="F134:F140" si="186">$E$16/I134</f>
+        <v>14.21875</v>
+      </c>
+      <c r="G134">
+        <f t="shared" ref="G134:G140" si="187">G133+H134</f>
+        <v>1179648</v>
+      </c>
+      <c r="H134">
+        <f t="shared" ref="H134" si="188">H126*2</f>
+        <v>131072</v>
+      </c>
+      <c r="I134">
+        <f t="shared" si="130"/>
+        <v>288</v>
+      </c>
+      <c r="J134">
+        <f t="shared" si="182"/>
+        <v>1179648</v>
+      </c>
+      <c r="K134">
+        <f t="shared" ref="K134:K140" si="189">FLOOR(J134/G134,1)</f>
+        <v>1</v>
+      </c>
+      <c r="L134" s="1">
+        <f t="shared" ref="L134:L140" si="190">(J134-K134*G134)/J134</f>
+        <v>0</v>
+      </c>
+      <c r="M134" s="1">
+        <f t="shared" ref="M134:M140" si="191">(G134-(G133+1))/(G134)</f>
+        <v>0.11111026340060765</v>
+      </c>
+      <c r="N134">
+        <f t="shared" ref="N134:N140" si="192">J134/4096</f>
+        <v>288</v>
+      </c>
+      <c r="O134">
+        <f t="shared" si="111"/>
+        <v>65536</v>
+      </c>
+      <c r="P134">
+        <f t="shared" si="183"/>
+        <v>0</v>
+      </c>
+      <c r="Q134">
+        <f t="shared" ref="Q134:Q140" si="193">P134/I134</f>
+        <v>0</v>
+      </c>
+      <c r="S134">
+        <f t="shared" si="184"/>
+        <v>0</v>
+      </c>
+      <c r="AC134" s="1"/>
+      <c r="AD134" s="1"/>
+    </row>
+    <row r="135" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D135">
+        <f t="shared" ref="D135:D140" si="194">I135/5</f>
+        <v>64</v>
+      </c>
+      <c r="E135" s="1">
+        <f t="shared" si="180"/>
+        <v>6.2271062271062272E-2</v>
+      </c>
+      <c r="F135">
+        <f t="shared" ref="F135:F140" si="195">$E$17/I135</f>
+        <v>12.796875</v>
+      </c>
+      <c r="G135">
+        <f t="shared" si="187"/>
+        <v>1310720</v>
+      </c>
+      <c r="H135">
+        <f t="shared" si="95"/>
+        <v>131072</v>
+      </c>
+      <c r="I135">
+        <f t="shared" si="130"/>
+        <v>320</v>
+      </c>
+      <c r="J135">
+        <f t="shared" si="182"/>
+        <v>1310720</v>
+      </c>
+      <c r="K135">
+        <f t="shared" si="189"/>
+        <v>1</v>
+      </c>
+      <c r="L135" s="1">
+        <f t="shared" si="190"/>
+        <v>0</v>
+      </c>
+      <c r="M135" s="1">
+        <f t="shared" si="191"/>
+        <v>9.9999237060546878E-2</v>
+      </c>
+      <c r="N135">
+        <f t="shared" si="192"/>
+        <v>320</v>
+      </c>
+      <c r="O135">
+        <f t="shared" si="111"/>
+        <v>131072</v>
+      </c>
+      <c r="P135">
+        <f t="shared" si="183"/>
+        <v>0</v>
+      </c>
+      <c r="Q135">
+        <f t="shared" si="193"/>
+        <v>0</v>
+      </c>
+      <c r="S135">
+        <f t="shared" si="184"/>
+        <v>0</v>
+      </c>
+      <c r="AC135" s="1"/>
+      <c r="AD135" s="1"/>
+    </row>
+    <row r="136" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D136">
+        <f t="shared" ref="D136:D140" si="196">I136/11</f>
+        <v>32</v>
+      </c>
+      <c r="E136" s="1">
+        <f t="shared" si="180"/>
+        <v>5.3763440860215055E-2</v>
+      </c>
+      <c r="F136">
+        <f t="shared" ref="F136:F140" si="197">$E$18/I136</f>
+        <v>11.625</v>
+      </c>
+      <c r="G136">
+        <f t="shared" si="187"/>
+        <v>1441792</v>
+      </c>
+      <c r="H136">
+        <f t="shared" si="95"/>
+        <v>131072</v>
+      </c>
+      <c r="I136">
+        <f t="shared" si="130"/>
+        <v>352</v>
+      </c>
+      <c r="J136">
+        <f t="shared" si="182"/>
+        <v>1441792</v>
+      </c>
+      <c r="K136">
+        <f t="shared" si="189"/>
+        <v>1</v>
+      </c>
+      <c r="L136" s="1">
+        <f t="shared" si="190"/>
+        <v>0</v>
+      </c>
+      <c r="M136" s="1">
+        <f t="shared" si="191"/>
+        <v>9.0908397327769883E-2</v>
+      </c>
+      <c r="N136">
+        <f t="shared" si="192"/>
+        <v>352</v>
+      </c>
+      <c r="O136">
+        <f t="shared" si="111"/>
+        <v>65536</v>
+      </c>
+      <c r="P136">
+        <f t="shared" si="183"/>
+        <v>0</v>
+      </c>
+      <c r="Q136">
+        <f t="shared" si="193"/>
+        <v>0</v>
+      </c>
+      <c r="S136">
+        <f t="shared" si="184"/>
+        <v>0</v>
+      </c>
+      <c r="AC136" s="1"/>
+      <c r="AD136" s="1"/>
+    </row>
+    <row r="137" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D137">
+        <f t="shared" ref="D137:D140" si="198">I137/3</f>
+        <v>128</v>
+      </c>
+      <c r="E137" s="1">
+        <f t="shared" si="180"/>
+        <v>6.2271062271062272E-2</v>
+      </c>
+      <c r="F137">
+        <f t="shared" ref="F137:F140" si="199">$E$19/I137</f>
+        <v>10.6640625</v>
+      </c>
+      <c r="G137">
+        <f t="shared" si="187"/>
+        <v>1572864</v>
+      </c>
+      <c r="H137">
+        <f t="shared" si="95"/>
+        <v>131072</v>
+      </c>
+      <c r="I137">
+        <f t="shared" si="130"/>
+        <v>384</v>
+      </c>
+      <c r="J137">
+        <f t="shared" si="182"/>
+        <v>1572864</v>
+      </c>
+      <c r="K137">
+        <f t="shared" si="189"/>
+        <v>1</v>
+      </c>
+      <c r="L137" s="1">
+        <f t="shared" si="190"/>
+        <v>0</v>
+      </c>
+      <c r="M137" s="1">
+        <f t="shared" si="191"/>
+        <v>8.3332697550455734E-2</v>
+      </c>
+      <c r="N137">
+        <f t="shared" si="192"/>
+        <v>384</v>
+      </c>
+      <c r="O137">
+        <f t="shared" si="111"/>
+        <v>262144</v>
+      </c>
+      <c r="P137">
+        <f t="shared" si="183"/>
+        <v>0</v>
+      </c>
+      <c r="Q137">
+        <f t="shared" si="193"/>
+        <v>0</v>
+      </c>
+      <c r="S137">
+        <f t="shared" si="184"/>
+        <v>0</v>
+      </c>
+      <c r="AC137" s="1"/>
+      <c r="AD137" s="1"/>
+    </row>
+    <row r="138" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D138">
+        <f t="shared" ref="D138:D140" si="200">I138/13</f>
+        <v>32</v>
+      </c>
+      <c r="E138" s="1">
+        <f t="shared" si="180"/>
+        <v>8.5714285714285715E-2</v>
+      </c>
+      <c r="F138">
+        <f t="shared" ref="F138:F140" si="201">$E$20/I138</f>
+        <v>9.84375</v>
+      </c>
+      <c r="G138">
+        <f t="shared" si="187"/>
+        <v>1703936</v>
+      </c>
+      <c r="H138">
+        <f t="shared" si="95"/>
+        <v>131072</v>
+      </c>
+      <c r="I138">
+        <f t="shared" si="130"/>
+        <v>416</v>
+      </c>
+      <c r="J138">
+        <f t="shared" si="182"/>
+        <v>1703936</v>
+      </c>
+      <c r="K138">
+        <f t="shared" si="189"/>
+        <v>1</v>
+      </c>
+      <c r="L138" s="1">
+        <f t="shared" si="190"/>
+        <v>0</v>
+      </c>
+      <c r="M138" s="1">
+        <f t="shared" si="191"/>
+        <v>7.6922490046574518E-2</v>
+      </c>
+      <c r="N138">
+        <f t="shared" si="192"/>
+        <v>416</v>
+      </c>
+      <c r="O138">
+        <f t="shared" si="111"/>
+        <v>65536</v>
+      </c>
+      <c r="P138">
+        <f t="shared" si="183"/>
+        <v>0</v>
+      </c>
+      <c r="Q138">
+        <f t="shared" si="193"/>
+        <v>0</v>
+      </c>
+      <c r="S138">
+        <f t="shared" si="184"/>
+        <v>0</v>
+      </c>
+      <c r="AC138" s="1"/>
+      <c r="AD138" s="1"/>
+    </row>
+    <row r="139" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D139">
+        <f t="shared" ref="D139:D140" si="202">I139/7</f>
+        <v>64</v>
+      </c>
+      <c r="E139" s="1">
+        <f t="shared" si="180"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="F139">
+        <f t="shared" ref="F139:F140" si="203">$E$21/I139</f>
+        <v>9.140625</v>
+      </c>
+      <c r="G139">
+        <f t="shared" si="187"/>
+        <v>1835008</v>
+      </c>
+      <c r="H139">
+        <f t="shared" si="95"/>
+        <v>131072</v>
+      </c>
+      <c r="I139">
+        <f t="shared" si="130"/>
+        <v>448</v>
+      </c>
+      <c r="J139">
+        <f t="shared" si="182"/>
+        <v>1835008</v>
+      </c>
+      <c r="K139">
+        <f t="shared" si="189"/>
+        <v>1</v>
+      </c>
+      <c r="L139" s="1">
+        <f t="shared" si="190"/>
+        <v>0</v>
+      </c>
+      <c r="M139" s="1">
+        <f t="shared" si="191"/>
+        <v>7.14280264718192E-2</v>
+      </c>
+      <c r="N139">
+        <f t="shared" si="192"/>
+        <v>448</v>
+      </c>
+      <c r="O139">
+        <f t="shared" si="111"/>
+        <v>131072</v>
+      </c>
+      <c r="P139">
+        <f t="shared" si="183"/>
+        <v>0</v>
+      </c>
+      <c r="Q139">
+        <f t="shared" si="193"/>
+        <v>0</v>
+      </c>
+      <c r="S139">
+        <f t="shared" si="184"/>
+        <v>0</v>
+      </c>
+      <c r="AC139" s="1"/>
+      <c r="AD139" s="1"/>
+    </row>
+    <row r="140" spans="4:30" x14ac:dyDescent="0.2">
+      <c r="D140">
+        <f t="shared" ref="D140" si="204">I140/15</f>
+        <v>32</v>
+      </c>
+      <c r="E140" s="1">
+        <f t="shared" si="180"/>
+        <v>6.2271062271062272E-2</v>
+      </c>
+      <c r="F140">
+        <f t="shared" ref="F140" si="205">$E$22/I140</f>
+        <v>8.53125</v>
+      </c>
+      <c r="G140">
+        <f t="shared" si="187"/>
+        <v>1966080</v>
+      </c>
+      <c r="H140">
+        <f t="shared" si="95"/>
+        <v>131072</v>
+      </c>
+      <c r="I140">
+        <f t="shared" si="130"/>
+        <v>480</v>
+      </c>
+      <c r="J140">
+        <f t="shared" si="182"/>
+        <v>1966080</v>
+      </c>
+      <c r="K140">
+        <f t="shared" si="189"/>
+        <v>1</v>
+      </c>
+      <c r="L140" s="1">
+        <f t="shared" si="190"/>
+        <v>0</v>
+      </c>
+      <c r="M140" s="1">
+        <f t="shared" si="191"/>
+        <v>6.666615804036459E-2</v>
+      </c>
+      <c r="N140">
+        <f t="shared" si="192"/>
+        <v>480</v>
+      </c>
+      <c r="O140">
+        <f t="shared" si="111"/>
+        <v>65536</v>
+      </c>
+      <c r="P140">
+        <f t="shared" si="183"/>
+        <v>0</v>
+      </c>
+      <c r="Q140">
+        <f t="shared" si="193"/>
+        <v>0</v>
+      </c>
+      <c r="S140">
+        <f t="shared" si="184"/>
+        <v>0</v>
+      </c>
+      <c r="AC140" s="1"/>
+      <c r="AD140" s="1"/>
+    </row>
+    <row r="141" spans="4:30" x14ac:dyDescent="0.2">
       <c r="E141" s="1"/>
       <c r="L141" s="1"/>
       <c r="M141" s="1"/>
-    </row>
-    <row r="142" spans="5:13">
+      <c r="AC141" s="1"/>
+      <c r="AD141" s="1"/>
+    </row>
+    <row r="142" spans="4:30" x14ac:dyDescent="0.2">
       <c r="E142" s="1"/>
       <c r="L142" s="1"/>
       <c r="M142" s="1"/>
-    </row>
-    <row r="143" spans="5:13">
+      <c r="AC142" s="1"/>
+      <c r="AD142" s="1"/>
+    </row>
+    <row r="143" spans="4:30" x14ac:dyDescent="0.2">
       <c r="E143" s="1"/>
       <c r="L143" s="1"/>
       <c r="M143" s="1"/>
-    </row>
-    <row r="144" spans="5:13">
+      <c r="AC143" s="1"/>
+      <c r="AD143" s="1"/>
+    </row>
+    <row r="144" spans="4:30" x14ac:dyDescent="0.2">
       <c r="E144" s="1"/>
       <c r="L144" s="1"/>
       <c r="M144" s="1"/>
-    </row>
-    <row r="145" spans="5:13">
+      <c r="AC144" s="1"/>
+      <c r="AD144" s="1"/>
+    </row>
+    <row r="145" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E145" s="1"/>
       <c r="L145" s="1"/>
       <c r="M145" s="1"/>
-    </row>
-    <row r="146" spans="5:13">
+      <c r="AC145" s="1"/>
+      <c r="AD145" s="1"/>
+    </row>
+    <row r="146" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E146" s="1"/>
       <c r="L146" s="1"/>
       <c r="M146" s="1"/>
-    </row>
-    <row r="147" spans="5:13">
+      <c r="AC146" s="1"/>
+      <c r="AD146" s="1"/>
+    </row>
+    <row r="147" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E147" s="1"/>
       <c r="L147" s="1"/>
       <c r="M147" s="1"/>
-    </row>
-    <row r="148" spans="5:13">
+      <c r="AC147" s="1"/>
+      <c r="AD147" s="1"/>
+    </row>
+    <row r="148" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E148" s="1"/>
       <c r="L148" s="1"/>
       <c r="M148" s="1"/>
-    </row>
-    <row r="149" spans="5:13">
+      <c r="AC148" s="1"/>
+      <c r="AD148" s="1"/>
+    </row>
+    <row r="149" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E149" s="1"/>
       <c r="L149" s="1"/>
       <c r="M149" s="1"/>
-    </row>
-    <row r="150" spans="5:13">
+      <c r="AC149" s="1"/>
+      <c r="AD149" s="1"/>
+    </row>
+    <row r="150" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E150" s="1"/>
       <c r="L150" s="1"/>
       <c r="M150" s="1"/>
-    </row>
-    <row r="151" spans="5:13">
+      <c r="AC150" s="1"/>
+      <c r="AD150" s="1"/>
+    </row>
+    <row r="151" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E151" s="1"/>
       <c r="L151" s="1"/>
       <c r="M151" s="1"/>
-    </row>
-    <row r="152" spans="5:13">
+      <c r="AC151" s="1"/>
+      <c r="AD151" s="1"/>
+    </row>
+    <row r="152" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E152" s="1"/>
       <c r="L152" s="1"/>
       <c r="M152" s="1"/>
-    </row>
-    <row r="153" spans="5:13">
+      <c r="AC152" s="1"/>
+      <c r="AD152" s="1"/>
+    </row>
+    <row r="153" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E153" s="1"/>
       <c r="L153" s="1"/>
       <c r="M153" s="1"/>
-    </row>
-    <row r="154" spans="5:13">
+      <c r="AC153" s="1"/>
+      <c r="AD153" s="1"/>
+    </row>
+    <row r="154" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E154" s="1"/>
       <c r="L154" s="1"/>
       <c r="M154" s="1"/>
-    </row>
-    <row r="155" spans="5:13">
+      <c r="AC154" s="1"/>
+      <c r="AD154" s="1"/>
+    </row>
+    <row r="155" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E155" s="1"/>
       <c r="L155" s="1"/>
       <c r="M155" s="1"/>
     </row>
-    <row r="156" spans="5:13">
+    <row r="156" spans="3:30" x14ac:dyDescent="0.2">
+      <c r="C156" t="s">
+        <v>8</v>
+      </c>
       <c r="E156" s="1"/>
       <c r="L156" s="1"/>
-      <c r="M156" s="1"/>
-    </row>
-    <row r="157" spans="5:13">
+      <c r="M156" s="1">
+        <f>MAX(M13:M140)</f>
+        <v>0.11111026340060765</v>
+      </c>
+    </row>
+    <row r="157" spans="3:30" x14ac:dyDescent="0.2">
+      <c r="C157" t="s">
+        <v>9</v>
+      </c>
       <c r="E157" s="1"/>
       <c r="L157" s="1"/>
-      <c r="M157" s="1"/>
-    </row>
-    <row r="158" spans="5:13">
+      <c r="M157" s="1">
+        <f>AVERAGE(M13:M140)</f>
+        <v>8.0513821991497744E-2</v>
+      </c>
+    </row>
+    <row r="158" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E158" s="1"/>
       <c r="L158" s="1"/>
       <c r="M158" s="1"/>
     </row>
-    <row r="159" spans="5:13">
+    <row r="159" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E159" s="1"/>
       <c r="L159" s="1"/>
       <c r="M159" s="1"/>
     </row>
-    <row r="160" spans="5:13">
+    <row r="160" spans="3:30" x14ac:dyDescent="0.2">
       <c r="E160" s="1"/>
       <c r="L160" s="1"/>
       <c r="M160" s="1"/>
     </row>
-    <row r="161" spans="5:13">
+    <row r="161" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E161" s="1"/>
       <c r="L161" s="1"/>
       <c r="M161" s="1"/>
     </row>
-    <row r="162" spans="5:13">
+    <row r="162" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E162" s="1"/>
       <c r="L162" s="1"/>
       <c r="M162" s="1"/>
     </row>
-    <row r="163" spans="5:13">
+    <row r="163" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E163" s="1"/>
       <c r="L163" s="1"/>
       <c r="M163" s="1"/>
     </row>
-    <row r="164" spans="5:13">
+    <row r="164" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E164" s="1"/>
       <c r="L164" s="1"/>
       <c r="M164" s="1"/>
     </row>
-    <row r="165" spans="5:13">
+    <row r="165" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E165" s="1"/>
       <c r="L165" s="1"/>
       <c r="M165" s="1"/>
     </row>
-    <row r="166" spans="5:13">
+    <row r="166" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E166" s="1"/>
       <c r="L166" s="1"/>
       <c r="M166" s="1"/>
     </row>
-    <row r="167" spans="5:13">
+    <row r="167" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E167" s="1"/>
       <c r="L167" s="1"/>
       <c r="M167" s="1"/>
     </row>
-    <row r="168" spans="5:13">
+    <row r="168" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E168" s="1"/>
       <c r="L168" s="1"/>
       <c r="M168" s="1"/>
     </row>
-    <row r="169" spans="5:13">
+    <row r="169" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E169" s="1"/>
       <c r="L169" s="1"/>
       <c r="M169" s="1"/>
     </row>
-    <row r="170" spans="5:13">
+    <row r="170" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E170" s="1"/>
       <c r="L170" s="1"/>
       <c r="M170" s="1"/>
     </row>
-    <row r="171" spans="5:13">
+    <row r="171" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E171" s="1"/>
       <c r="L171" s="1"/>
       <c r="M171" s="1"/>
     </row>
-    <row r="172" spans="5:13">
+    <row r="172" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E172" s="1"/>
       <c r="L172" s="1"/>
       <c r="M172" s="1"/>
     </row>
-    <row r="173" spans="5:13">
+    <row r="173" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E173" s="1"/>
       <c r="L173" s="1"/>
       <c r="M173" s="1"/>
     </row>
-    <row r="174" spans="5:13">
+    <row r="174" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E174" s="1"/>
       <c r="L174" s="1"/>
       <c r="M174" s="1"/>
     </row>
-    <row r="175" spans="5:13">
+    <row r="175" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E175" s="1"/>
       <c r="L175" s="1"/>
       <c r="M175" s="1"/>
     </row>
-    <row r="176" spans="5:13">
+    <row r="176" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E176" s="1"/>
       <c r="L176" s="1"/>
       <c r="M176" s="1"/>
     </row>
-    <row r="177" spans="5:13">
+    <row r="177" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E177" s="1"/>
       <c r="L177" s="1"/>
       <c r="M177" s="1"/>
     </row>
-    <row r="178" spans="5:13">
+    <row r="178" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E178" s="1"/>
       <c r="L178" s="1"/>
       <c r="M178" s="1"/>
     </row>
-    <row r="179" spans="5:13">
+    <row r="179" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E179" s="1"/>
       <c r="L179" s="1"/>
       <c r="M179" s="1"/>
     </row>
-    <row r="180" spans="5:13">
+    <row r="180" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E180" s="1"/>
       <c r="L180" s="1"/>
       <c r="M180" s="1"/>
     </row>
-    <row r="181" spans="5:13">
+    <row r="181" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E181" s="1"/>
       <c r="L181" s="1"/>
       <c r="M181" s="1"/>
     </row>
-    <row r="182" spans="5:13">
+    <row r="182" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E182" s="1"/>
       <c r="L182" s="1"/>
       <c r="M182" s="1"/>
     </row>
-    <row r="183" spans="5:13">
+    <row r="183" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E183" s="1"/>
       <c r="L183" s="1"/>
       <c r="M183" s="1"/>
     </row>
-    <row r="184" spans="5:13">
+    <row r="184" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E184" s="1"/>
       <c r="L184" s="1"/>
       <c r="M184" s="1"/>
     </row>
-    <row r="185" spans="5:13">
+    <row r="185" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E185" s="1"/>
       <c r="L185" s="1"/>
       <c r="M185" s="1"/>
     </row>
-    <row r="186" spans="5:13">
+    <row r="186" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E186" s="1"/>
       <c r="L186" s="1"/>
       <c r="M186" s="1"/>
     </row>
-    <row r="187" spans="5:13">
+    <row r="187" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E187" s="1"/>
       <c r="L187" s="1"/>
       <c r="M187" s="1"/>
     </row>
-    <row r="188" spans="5:13">
+    <row r="188" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E188" s="1"/>
       <c r="L188" s="1"/>
       <c r="M188" s="1"/>
     </row>
-    <row r="189" spans="5:13">
+    <row r="189" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E189" s="1"/>
       <c r="L189" s="1"/>
       <c r="M189" s="1"/>
     </row>
-    <row r="190" spans="5:13">
+    <row r="190" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E190" s="1"/>
       <c r="L190" s="1"/>
       <c r="M190" s="1"/>
     </row>
-    <row r="191" spans="5:13">
+    <row r="191" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E191" s="1"/>
       <c r="L191" s="1"/>
       <c r="M191" s="1"/>
     </row>
-    <row r="192" spans="5:13">
+    <row r="192" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E192" s="1"/>
       <c r="L192" s="1"/>
       <c r="M192" s="1"/>
     </row>
-    <row r="193" spans="5:13">
+    <row r="193" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E193" s="1"/>
       <c r="L193" s="1"/>
       <c r="M193" s="1"/>
     </row>
-    <row r="194" spans="5:13">
+    <row r="194" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E194" s="1"/>
       <c r="L194" s="1"/>
       <c r="M194" s="1"/>
     </row>
-    <row r="195" spans="5:13">
+    <row r="195" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E195" s="1"/>
       <c r="L195" s="1"/>
       <c r="M195" s="1"/>
     </row>
-    <row r="196" spans="5:13">
+    <row r="196" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E196" s="1"/>
       <c r="L196" s="1"/>
       <c r="M196" s="1"/>
     </row>
-    <row r="197" spans="5:13">
+    <row r="197" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E197" s="1"/>
       <c r="L197" s="1"/>
       <c r="M197" s="1"/>
     </row>
-    <row r="198" spans="5:13">
+    <row r="198" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E198" s="1"/>
       <c r="L198" s="1"/>
       <c r="M198" s="1"/>
     </row>
-    <row r="199" spans="5:13">
+    <row r="199" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E199" s="1"/>
       <c r="L199" s="1"/>
       <c r="M199" s="1"/>
     </row>
-    <row r="200" spans="5:13">
+    <row r="200" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E200" s="1"/>
       <c r="L200" s="1"/>
       <c r="M200" s="1"/>
     </row>
-    <row r="201" spans="5:13">
+    <row r="201" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E201" s="1"/>
       <c r="L201" s="1"/>
       <c r="M201" s="1"/>
     </row>
-    <row r="202" spans="5:13">
+    <row r="202" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E202" s="1"/>
       <c r="L202" s="1"/>
       <c r="M202" s="1"/>
     </row>
-    <row r="203" spans="5:13">
+    <row r="203" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E203" s="1"/>
       <c r="L203" s="1"/>
       <c r="M203" s="1"/>
     </row>
-    <row r="204" spans="5:13">
+    <row r="204" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E204" s="1"/>
       <c r="L204" s="1"/>
       <c r="M204" s="1"/>
     </row>
-    <row r="205" spans="5:13">
+    <row r="205" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E205" s="1"/>
       <c r="L205" s="1"/>
       <c r="M205" s="1"/>
     </row>
-    <row r="206" spans="5:13">
+    <row r="206" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E206" s="1"/>
       <c r="L206" s="1"/>
       <c r="M206" s="1"/>
     </row>
-    <row r="207" spans="5:13">
+    <row r="207" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E207" s="1"/>
       <c r="L207" s="1"/>
       <c r="M207" s="1"/>
     </row>
-    <row r="208" spans="5:13">
+    <row r="208" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E208" s="1"/>
       <c r="L208" s="1"/>
       <c r="M208" s="1"/>
     </row>
-    <row r="209" spans="5:13">
+    <row r="209" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E209" s="1"/>
       <c r="L209" s="1"/>
       <c r="M209" s="1"/>
     </row>
-    <row r="210" spans="5:13">
+    <row r="210" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E210" s="1"/>
       <c r="L210" s="1"/>
       <c r="M210" s="1"/>
     </row>
-    <row r="211" spans="5:13">
+    <row r="211" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E211" s="1"/>
       <c r="L211" s="1"/>
       <c r="M211" s="1"/>
     </row>
-    <row r="212" spans="5:13">
+    <row r="212" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E212" s="1"/>
       <c r="L212" s="1"/>
       <c r="M212" s="1"/>
     </row>
-    <row r="213" spans="5:13">
+    <row r="213" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E213" s="1"/>
       <c r="L213" s="1"/>
       <c r="M213" s="1"/>
     </row>
-    <row r="214" spans="5:13">
+    <row r="214" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E214" s="1"/>
       <c r="L214" s="1"/>
       <c r="M214" s="1"/>
     </row>
-    <row r="215" spans="5:13">
+    <row r="215" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E215" s="1"/>
       <c r="L215" s="1"/>
       <c r="M215" s="1"/>
     </row>
-    <row r="216" spans="5:13">
+    <row r="216" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E216" s="1"/>
       <c r="L216" s="1"/>
       <c r="M216" s="1"/>
     </row>
-    <row r="217" spans="5:13">
+    <row r="217" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E217" s="1"/>
       <c r="L217" s="1"/>
       <c r="M217" s="1"/>
     </row>
-    <row r="218" spans="5:13">
+    <row r="218" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E218" s="1"/>
       <c r="L218" s="1"/>
       <c r="M218" s="1"/>
     </row>
-    <row r="219" spans="5:13">
+    <row r="219" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E219" s="1"/>
       <c r="L219" s="1"/>
       <c r="M219" s="1"/>
     </row>
-    <row r="220" spans="5:13">
+    <row r="220" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E220" s="1"/>
       <c r="L220" s="1"/>
       <c r="M220" s="1"/>
     </row>
-    <row r="221" spans="5:13">
+    <row r="221" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E221" s="1"/>
       <c r="L221" s="1"/>
       <c r="M221" s="1"/>
     </row>
-    <row r="222" spans="5:13">
+    <row r="222" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E222" s="1"/>
       <c r="L222" s="1"/>
       <c r="M222" s="1"/>
     </row>
-    <row r="223" spans="5:13">
+    <row r="223" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E223" s="1"/>
       <c r="L223" s="1"/>
       <c r="M223" s="1"/>
     </row>
-    <row r="224" spans="5:13">
+    <row r="224" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E224" s="1"/>
       <c r="L224" s="1"/>
       <c r="M224" s="1"/>
     </row>
-    <row r="225" spans="5:13">
+    <row r="225" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E225" s="1"/>
       <c r="L225" s="1"/>
       <c r="M225" s="1"/>
     </row>
-    <row r="226" spans="5:13">
+    <row r="226" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E226" s="1"/>
       <c r="L226" s="1"/>
       <c r="M226" s="1"/>
     </row>
-    <row r="227" spans="5:13">
+    <row r="227" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E227" s="1"/>
       <c r="L227" s="1"/>
       <c r="M227" s="1"/>
     </row>
-    <row r="228" spans="5:13">
+    <row r="228" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E228" s="1"/>
       <c r="L228" s="1"/>
       <c r="M228" s="1"/>
     </row>
-    <row r="229" spans="5:13">
+    <row r="229" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E229" s="1"/>
       <c r="L229" s="1"/>
       <c r="M229" s="1"/>
     </row>
-    <row r="230" spans="5:13">
+    <row r="230" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E230" s="1"/>
       <c r="L230" s="1"/>
       <c r="M230" s="1"/>
     </row>
-    <row r="231" spans="5:13">
+    <row r="231" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E231" s="1"/>
       <c r="L231" s="1"/>
       <c r="M231" s="1"/>
     </row>
-    <row r="232" spans="5:13">
+    <row r="232" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E232" s="1"/>
       <c r="L232" s="1"/>
       <c r="M232" s="1"/>
     </row>
-    <row r="233" spans="5:13">
+    <row r="233" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E233" s="1"/>
       <c r="L233" s="1"/>
       <c r="M233" s="1"/>
     </row>
-    <row r="234" spans="5:13">
+    <row r="234" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E234" s="1"/>
       <c r="L234" s="1"/>
       <c r="M234" s="1"/>
     </row>
-    <row r="235" spans="5:13">
+    <row r="235" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E235" s="1"/>
       <c r="L235" s="1"/>
       <c r="M235" s="1"/>
     </row>
-    <row r="236" spans="5:13">
+    <row r="236" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E236" s="1"/>
       <c r="L236" s="1"/>
       <c r="M236" s="1"/>
     </row>
-    <row r="237" spans="5:13">
+    <row r="237" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E237" s="1"/>
       <c r="L237" s="1"/>
       <c r="M237" s="1"/>
     </row>
-    <row r="238" spans="5:13">
+    <row r="238" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E238" s="1"/>
       <c r="L238" s="1"/>
       <c r="M238" s="1"/>
     </row>
-    <row r="239" spans="5:13">
+    <row r="239" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E239" s="1"/>
       <c r="L239" s="1"/>
       <c r="M239" s="1"/>
     </row>
-    <row r="240" spans="5:13">
+    <row r="240" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E240" s="1"/>
       <c r="L240" s="1"/>
       <c r="M240" s="1"/>
     </row>
-    <row r="241" spans="5:13">
+    <row r="241" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E241" s="1"/>
       <c r="L241" s="1"/>
       <c r="M241" s="1"/>
     </row>
-    <row r="242" spans="5:13">
+    <row r="242" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E242" s="1"/>
       <c r="L242" s="1"/>
       <c r="M242" s="1"/>
     </row>
-    <row r="243" spans="5:13">
+    <row r="243" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E243" s="1"/>
       <c r="L243" s="1"/>
       <c r="M243" s="1"/>
     </row>
-    <row r="244" spans="5:13">
+    <row r="244" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E244" s="1"/>
       <c r="L244" s="1"/>
       <c r="M244" s="1"/>
     </row>
-    <row r="245" spans="5:13">
+    <row r="245" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E245" s="1"/>
       <c r="L245" s="1"/>
       <c r="M245" s="1"/>
     </row>
-    <row r="246" spans="5:13">
+    <row r="246" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E246" s="1"/>
       <c r="L246" s="1"/>
       <c r="M246" s="1"/>
     </row>
-    <row r="247" spans="5:13">
+    <row r="247" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E247" s="1"/>
       <c r="L247" s="1"/>
       <c r="M247" s="1"/>
     </row>
-    <row r="248" spans="5:13">
+    <row r="248" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E248" s="1"/>
       <c r="L248" s="1"/>
       <c r="M248" s="1"/>
     </row>
-    <row r="249" spans="5:13">
+    <row r="249" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E249" s="1"/>
       <c r="L249" s="1"/>
       <c r="M249" s="1"/>
     </row>
-    <row r="250" spans="5:13">
+    <row r="250" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E250" s="1"/>
       <c r="L250" s="1"/>
       <c r="M250" s="1"/>
     </row>
-    <row r="251" spans="5:13">
+    <row r="251" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E251" s="1"/>
       <c r="L251" s="1"/>
       <c r="M251" s="1"/>
     </row>
-    <row r="252" spans="5:13">
+    <row r="252" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E252" s="1"/>
       <c r="L252" s="1"/>
       <c r="M252" s="1"/>
     </row>
-    <row r="253" spans="5:13">
+    <row r="253" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E253" s="1"/>
       <c r="L253" s="1"/>
       <c r="M253" s="1"/>
     </row>
-    <row r="254" spans="5:13">
+    <row r="254" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E254" s="1"/>
       <c r="L254" s="1"/>
       <c r="M254" s="1"/>
     </row>
-    <row r="255" spans="5:13">
+    <row r="255" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E255" s="1"/>
       <c r="L255" s="1"/>
       <c r="M255" s="1"/>
     </row>
-    <row r="256" spans="5:13">
+    <row r="256" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E256" s="1"/>
       <c r="L256" s="1"/>
       <c r="M256" s="1"/>
     </row>
-    <row r="257" spans="5:13">
+    <row r="257" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E257" s="1"/>
       <c r="L257" s="1"/>
       <c r="M257" s="1"/>
     </row>
-    <row r="258" spans="5:13">
+    <row r="258" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E258" s="1"/>
       <c r="L258" s="1"/>
       <c r="M258" s="1"/>
     </row>
-    <row r="259" spans="5:13">
+    <row r="259" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E259" s="1"/>
       <c r="L259" s="1"/>
       <c r="M259" s="1"/>
     </row>
-    <row r="260" spans="5:13">
+    <row r="260" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E260" s="1"/>
       <c r="L260" s="1"/>
       <c r="M260" s="1"/>
     </row>
-    <row r="261" spans="5:13">
+    <row r="261" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E261" s="1"/>
       <c r="L261" s="1"/>
       <c r="M261" s="1"/>
     </row>
-    <row r="262" spans="5:13">
+    <row r="262" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E262" s="1"/>
       <c r="L262" s="1"/>
       <c r="M262" s="1"/>
     </row>
-    <row r="263" spans="5:13">
+    <row r="263" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E263" s="1"/>
       <c r="L263" s="1"/>
       <c r="M263" s="1"/>
     </row>
-    <row r="264" spans="5:13">
+    <row r="264" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E264" s="1"/>
       <c r="L264" s="1"/>
       <c r="M264" s="1"/>
     </row>
-    <row r="265" spans="5:13">
+    <row r="265" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E265" s="1"/>
       <c r="L265" s="1"/>
       <c r="M265" s="1"/>
     </row>
-    <row r="266" spans="5:13">
+    <row r="266" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E266" s="1"/>
       <c r="L266" s="1"/>
       <c r="M266" s="1"/>
     </row>
-    <row r="267" spans="5:13">
+    <row r="267" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E267" s="1"/>
       <c r="L267" s="1"/>
       <c r="M267" s="1"/>
     </row>
-    <row r="268" spans="5:13">
+    <row r="268" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E268" s="1"/>
       <c r="L268" s="1"/>
       <c r="M268" s="1"/>
     </row>
-    <row r="269" spans="5:13">
+    <row r="269" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E269" s="1"/>
       <c r="L269" s="1"/>
       <c r="M269" s="1"/>
     </row>
-    <row r="270" spans="5:13">
+    <row r="270" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E270" s="1"/>
       <c r="L270" s="1"/>
       <c r="M270" s="1"/>
     </row>
-    <row r="271" spans="5:13">
+    <row r="271" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E271" s="1"/>
       <c r="L271" s="1"/>
       <c r="M271" s="1"/>
     </row>
-    <row r="272" spans="5:13">
+    <row r="272" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E272" s="1"/>
       <c r="L272" s="1"/>
       <c r="M272" s="1"/>
     </row>
-    <row r="273" spans="5:13">
+    <row r="273" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E273" s="1"/>
       <c r="L273" s="1"/>
       <c r="M273" s="1"/>
     </row>
-    <row r="274" spans="5:13">
+    <row r="274" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E274" s="1"/>
       <c r="L274" s="1"/>
       <c r="M274" s="1"/>
     </row>
-    <row r="275" spans="5:13">
+    <row r="275" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E275" s="1"/>
       <c r="L275" s="1"/>
       <c r="M275" s="1"/>
     </row>
-    <row r="276" spans="5:13">
+    <row r="276" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E276" s="1"/>
       <c r="L276" s="1"/>
       <c r="M276" s="1"/>
     </row>
-    <row r="277" spans="5:13">
+    <row r="277" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E277" s="1"/>
       <c r="L277" s="1"/>
       <c r="M277" s="1"/>
     </row>
-    <row r="278" spans="5:13">
+    <row r="278" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E278" s="1"/>
       <c r="L278" s="1"/>
       <c r="M278" s="1"/>
     </row>
-    <row r="279" spans="5:13">
+    <row r="279" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E279" s="1"/>
       <c r="L279" s="1"/>
       <c r="M279" s="1"/>
     </row>
-    <row r="280" spans="5:13">
+    <row r="280" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E280" s="1"/>
       <c r="L280" s="1"/>
       <c r="M280" s="1"/>
     </row>
-    <row r="281" spans="5:13">
+    <row r="281" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E281" s="1"/>
       <c r="L281" s="1"/>
       <c r="M281" s="1"/>
     </row>
-    <row r="282" spans="5:13">
+    <row r="282" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E282" s="1"/>
       <c r="L282" s="1"/>
       <c r="M282" s="1"/>
     </row>
-    <row r="283" spans="5:13">
+    <row r="283" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E283" s="1"/>
       <c r="L283" s="1"/>
       <c r="M283" s="1"/>
     </row>
-    <row r="284" spans="5:13">
+    <row r="284" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E284" s="1"/>
       <c r="L284" s="1"/>
       <c r="M284" s="1"/>
     </row>
-    <row r="285" spans="5:13">
+    <row r="285" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E285" s="1"/>
       <c r="L285" s="1"/>
       <c r="M285" s="1"/>
     </row>
-    <row r="286" spans="5:13">
+    <row r="286" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E286" s="1"/>
       <c r="L286" s="1"/>
       <c r="M286" s="1"/>
     </row>
-    <row r="287" spans="5:13">
+    <row r="287" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E287" s="1"/>
       <c r="L287" s="1"/>
       <c r="M287" s="1"/>
     </row>
-    <row r="288" spans="5:13">
+    <row r="288" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E288" s="1"/>
       <c r="L288" s="1"/>
       <c r="M288" s="1"/>
     </row>
-    <row r="289" spans="5:13">
+    <row r="289" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E289" s="1"/>
       <c r="L289" s="1"/>
       <c r="M289" s="1"/>
     </row>
-    <row r="290" spans="5:13">
+    <row r="290" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E290" s="1"/>
       <c r="L290" s="1"/>
       <c r="M290" s="1"/>
     </row>
-    <row r="291" spans="5:13">
+    <row r="291" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E291" s="1"/>
       <c r="L291" s="1"/>
       <c r="M291" s="1"/>
     </row>
-    <row r="292" spans="5:13">
+    <row r="292" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E292" s="1"/>
       <c r="L292" s="1"/>
       <c r="M292" s="1"/>
     </row>
-    <row r="293" spans="5:13">
+    <row r="293" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E293" s="1"/>
       <c r="L293" s="1"/>
       <c r="M293" s="1"/>
     </row>
-    <row r="294" spans="5:13">
+    <row r="294" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E294" s="1"/>
       <c r="L294" s="1"/>
       <c r="M294" s="1"/>
     </row>
-    <row r="295" spans="5:13">
+    <row r="295" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E295" s="1"/>
       <c r="L295" s="1"/>
       <c r="M295" s="1"/>
     </row>
-    <row r="296" spans="5:13">
+    <row r="296" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E296" s="1"/>
       <c r="L296" s="1"/>
       <c r="M296" s="1"/>
     </row>
-    <row r="297" spans="5:13">
+    <row r="297" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E297" s="1"/>
       <c r="L297" s="1"/>
       <c r="M297" s="1"/>
     </row>
-    <row r="298" spans="5:13">
+    <row r="298" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E298" s="1"/>
       <c r="L298" s="1"/>
       <c r="M298" s="1"/>
     </row>
-    <row r="299" spans="5:13">
+    <row r="299" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E299" s="1"/>
       <c r="L299" s="1"/>
       <c r="M299" s="1"/>
     </row>
-    <row r="300" spans="5:13">
+    <row r="300" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E300" s="1"/>
       <c r="L300" s="1"/>
       <c r="M300" s="1"/>
     </row>
-    <row r="301" spans="5:13">
+    <row r="301" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E301" s="1"/>
       <c r="L301" s="1"/>
       <c r="M301" s="1"/>
     </row>
-    <row r="302" spans="5:13">
+    <row r="302" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E302" s="1"/>
       <c r="L302" s="1"/>
       <c r="M302" s="1"/>
     </row>
-    <row r="303" spans="5:13">
+    <row r="303" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E303" s="1"/>
       <c r="L303" s="1"/>
       <c r="M303" s="1"/>
     </row>
-    <row r="304" spans="5:13">
+    <row r="304" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E304" s="1"/>
       <c r="L304" s="1"/>
       <c r="M304" s="1"/>
     </row>
-    <row r="305" spans="5:13">
+    <row r="305" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E305" s="1"/>
       <c r="L305" s="1"/>
       <c r="M305" s="1"/>
     </row>
-    <row r="306" spans="5:13">
+    <row r="306" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E306" s="1"/>
       <c r="L306" s="1"/>
       <c r="M306" s="1"/>
     </row>
-    <row r="307" spans="5:13">
+    <row r="307" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E307" s="1"/>
       <c r="L307" s="1"/>
       <c r="M307" s="1"/>
     </row>
-    <row r="308" spans="5:13">
+    <row r="308" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E308" s="1"/>
       <c r="L308" s="1"/>
       <c r="M308" s="1"/>
     </row>
-    <row r="309" spans="5:13">
+    <row r="309" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E309" s="1"/>
       <c r="L309" s="1"/>
       <c r="M309" s="1"/>
     </row>
-    <row r="310" spans="5:13">
+    <row r="310" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E310" s="1"/>
       <c r="L310" s="1"/>
       <c r="M310" s="1"/>
     </row>
-    <row r="311" spans="5:13">
+    <row r="311" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E311" s="1"/>
       <c r="L311" s="1"/>
       <c r="M311" s="1"/>
     </row>
-    <row r="312" spans="5:13">
+    <row r="312" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E312" s="1"/>
       <c r="L312" s="1"/>
       <c r="M312" s="1"/>
     </row>
-    <row r="313" spans="5:13">
+    <row r="313" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E313" s="1"/>
       <c r="L313" s="1"/>
       <c r="M313" s="1"/>
     </row>
-    <row r="314" spans="5:13">
+    <row r="314" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E314" s="1"/>
       <c r="L314" s="1"/>
       <c r="M314" s="1"/>
     </row>
-    <row r="315" spans="5:13">
+    <row r="315" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E315" s="1"/>
       <c r="L315" s="1"/>
       <c r="M315" s="1"/>
     </row>
-    <row r="316" spans="5:13">
+    <row r="316" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E316" s="1"/>
       <c r="L316" s="1"/>
       <c r="M316" s="1"/>
     </row>
-    <row r="317" spans="5:13">
+    <row r="317" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E317" s="1"/>
       <c r="L317" s="1"/>
       <c r="M317" s="1"/>
     </row>
-    <row r="318" spans="5:13">
+    <row r="318" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E318" s="1"/>
       <c r="L318" s="1"/>
       <c r="M318" s="1"/>
     </row>
-    <row r="319" spans="5:13">
+    <row r="319" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E319" s="1"/>
       <c r="L319" s="1"/>
       <c r="M319" s="1"/>
     </row>
-    <row r="320" spans="5:13">
+    <row r="320" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E320" s="1"/>
       <c r="L320" s="1"/>
       <c r="M320" s="1"/>
     </row>
-    <row r="321" spans="5:13">
+    <row r="321" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E321" s="1"/>
       <c r="L321" s="1"/>
       <c r="M321" s="1"/>
     </row>
-    <row r="322" spans="5:13">
+    <row r="322" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E322" s="1"/>
       <c r="L322" s="1"/>
       <c r="M322" s="1"/>
     </row>
-    <row r="323" spans="5:13">
+    <row r="323" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E323" s="1"/>
       <c r="L323" s="1"/>
       <c r="M323" s="1"/>
     </row>
-    <row r="324" spans="5:13">
+    <row r="324" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E324" s="1"/>
       <c r="L324" s="1"/>
       <c r="M324" s="1"/>
     </row>
-    <row r="325" spans="5:13">
+    <row r="325" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E325" s="1"/>
       <c r="L325" s="1"/>
       <c r="M325" s="1"/>
     </row>
-    <row r="326" spans="5:13">
+    <row r="326" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E326" s="1"/>
       <c r="L326" s="1"/>
       <c r="M326" s="1"/>
     </row>
-    <row r="327" spans="5:13">
+    <row r="327" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E327" s="1"/>
       <c r="L327" s="1"/>
       <c r="M327" s="1"/>
     </row>
-    <row r="328" spans="5:13">
+    <row r="328" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E328" s="1"/>
       <c r="L328" s="1"/>
       <c r="M328" s="1"/>
     </row>
-    <row r="329" spans="5:13">
+    <row r="329" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E329" s="1"/>
       <c r="L329" s="1"/>
       <c r="M329" s="1"/>
     </row>
-    <row r="330" spans="5:13">
+    <row r="330" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E330" s="1"/>
       <c r="L330" s="1"/>
       <c r="M330" s="1"/>
     </row>
-    <row r="331" spans="5:13">
+    <row r="331" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E331" s="1"/>
       <c r="L331" s="1"/>
       <c r="M331" s="1"/>
     </row>
-    <row r="332" spans="5:13">
+    <row r="332" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E332" s="1"/>
       <c r="L332" s="1"/>
       <c r="M332" s="1"/>
     </row>
-    <row r="333" spans="5:13">
+    <row r="333" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E333" s="1"/>
       <c r="L333" s="1"/>
       <c r="M333" s="1"/>
     </row>
-    <row r="334" spans="5:13">
+    <row r="334" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E334" s="1"/>
       <c r="L334" s="1"/>
       <c r="M334" s="1"/>
     </row>
-    <row r="335" spans="5:13">
+    <row r="335" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E335" s="1"/>
       <c r="L335" s="1"/>
       <c r="M335" s="1"/>
     </row>
-    <row r="336" spans="5:13">
+    <row r="336" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E336" s="1"/>
       <c r="L336" s="1"/>
       <c r="M336" s="1"/>
     </row>
-    <row r="337" spans="5:13">
+    <row r="337" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E337" s="1"/>
       <c r="L337" s="1"/>
       <c r="M337" s="1"/>
     </row>
-    <row r="338" spans="5:13">
+    <row r="338" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E338" s="1"/>
       <c r="L338" s="1"/>
       <c r="M338" s="1"/>
     </row>
-    <row r="339" spans="5:13">
+    <row r="339" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E339" s="1"/>
       <c r="L339" s="1"/>
       <c r="M339" s="1"/>
     </row>
-    <row r="340" spans="5:13">
+    <row r="340" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E340" s="1"/>
       <c r="L340" s="1"/>
       <c r="M340" s="1"/>
     </row>
-    <row r="341" spans="5:13">
+    <row r="341" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E341" s="1"/>
       <c r="L341" s="1"/>
       <c r="M341" s="1"/>
     </row>
-    <row r="342" spans="5:13">
+    <row r="342" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E342" s="1"/>
       <c r="L342" s="1"/>
       <c r="M342" s="1"/>
     </row>
-    <row r="343" spans="5:13">
+    <row r="343" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E343" s="1"/>
       <c r="L343" s="1"/>
       <c r="M343" s="1"/>
     </row>
-    <row r="344" spans="5:13">
+    <row r="344" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E344" s="1"/>
       <c r="L344" s="1"/>
       <c r="M344" s="1"/>
     </row>
-    <row r="345" spans="5:13">
+    <row r="345" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E345" s="1"/>
       <c r="L345" s="1"/>
       <c r="M345" s="1"/>
     </row>
-    <row r="346" spans="5:13">
+    <row r="346" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E346" s="1"/>
       <c r="L346" s="1"/>
       <c r="M346" s="1"/>
     </row>
-    <row r="347" spans="5:13">
+    <row r="347" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E347" s="1"/>
       <c r="L347" s="1"/>
       <c r="M347" s="1"/>
     </row>
-    <row r="348" spans="5:13">
+    <row r="348" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E348" s="1"/>
       <c r="L348" s="1"/>
       <c r="M348" s="1"/>
     </row>
-    <row r="349" spans="5:13">
+    <row r="349" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E349" s="1"/>
       <c r="L349" s="1"/>
       <c r="M349" s="1"/>
     </row>
-    <row r="350" spans="5:13">
+    <row r="350" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E350" s="1"/>
       <c r="L350" s="1"/>
       <c r="M350" s="1"/>
     </row>
-    <row r="351" spans="5:13">
+    <row r="351" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E351" s="1"/>
       <c r="L351" s="1"/>
       <c r="M351" s="1"/>
     </row>
-    <row r="352" spans="5:13">
+    <row r="352" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E352" s="1"/>
       <c r="L352" s="1"/>
       <c r="M352" s="1"/>
     </row>
-    <row r="353" spans="5:13">
+    <row r="353" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E353" s="1"/>
       <c r="L353" s="1"/>
       <c r="M353" s="1"/>
     </row>
-    <row r="354" spans="5:13">
+    <row r="354" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E354" s="1"/>
       <c r="L354" s="1"/>
       <c r="M354" s="1"/>
     </row>
-    <row r="355" spans="5:13">
+    <row r="355" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E355" s="1"/>
       <c r="L355" s="1"/>
       <c r="M355" s="1"/>
     </row>
-    <row r="356" spans="5:13">
+    <row r="356" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E356" s="1"/>
       <c r="L356" s="1"/>
       <c r="M356" s="1"/>
     </row>
-    <row r="357" spans="5:13">
+    <row r="357" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E357" s="1"/>
       <c r="L357" s="1"/>
       <c r="M357" s="1"/>
     </row>
-    <row r="358" spans="5:13">
+    <row r="358" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E358" s="1"/>
       <c r="L358" s="1"/>
       <c r="M358" s="1"/>
     </row>
-    <row r="359" spans="5:13">
+    <row r="359" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E359" s="1"/>
       <c r="L359" s="1"/>
       <c r="M359" s="1"/>
     </row>
-    <row r="360" spans="5:13">
+    <row r="360" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E360" s="1"/>
       <c r="L360" s="1"/>
       <c r="M360" s="1"/>
     </row>
-    <row r="361" spans="5:13">
+    <row r="361" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E361" s="1"/>
       <c r="L361" s="1"/>
       <c r="M361" s="1"/>
     </row>
-    <row r="362" spans="5:13">
+    <row r="362" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E362" s="1"/>
       <c r="L362" s="1"/>
       <c r="M362" s="1"/>
     </row>
-    <row r="363" spans="5:13">
+    <row r="363" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E363" s="1"/>
       <c r="L363" s="1"/>
       <c r="M363" s="1"/>
     </row>
-    <row r="364" spans="5:13">
+    <row r="364" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E364" s="1"/>
       <c r="L364" s="1"/>
       <c r="M364" s="1"/>
     </row>
-    <row r="365" spans="5:13">
+    <row r="365" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E365" s="1"/>
       <c r="L365" s="1"/>
       <c r="M365" s="1"/>
     </row>
-    <row r="366" spans="5:13">
+    <row r="366" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E366" s="1"/>
       <c r="L366" s="1"/>
       <c r="M366" s="1"/>
     </row>
-    <row r="367" spans="5:13">
+    <row r="367" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E367" s="1"/>
       <c r="L367" s="1"/>
       <c r="M367" s="1"/>
     </row>
-    <row r="368" spans="5:13">
+    <row r="368" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E368" s="1"/>
       <c r="L368" s="1"/>
       <c r="M368" s="1"/>
     </row>
-    <row r="369" spans="5:13">
+    <row r="369" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E369" s="1"/>
       <c r="L369" s="1"/>
       <c r="M369" s="1"/>
     </row>
-    <row r="370" spans="5:13">
+    <row r="370" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E370" s="1"/>
       <c r="L370" s="1"/>
       <c r="M370" s="1"/>
     </row>
-    <row r="371" spans="5:13">
+    <row r="371" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E371" s="1"/>
       <c r="L371" s="1"/>
       <c r="M371" s="1"/>
     </row>
-    <row r="372" spans="5:13">
+    <row r="372" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E372" s="1"/>
       <c r="L372" s="1"/>
       <c r="M372" s="1"/>
     </row>
-    <row r="373" spans="5:13">
+    <row r="373" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E373" s="1"/>
       <c r="L373" s="1"/>
       <c r="M373" s="1"/>
     </row>
-    <row r="374" spans="5:13">
+    <row r="374" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E374" s="1"/>
       <c r="L374" s="1"/>
       <c r="M374" s="1"/>
     </row>
-    <row r="375" spans="5:13">
+    <row r="375" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E375" s="1"/>
       <c r="L375" s="1"/>
       <c r="M375" s="1"/>
     </row>
-    <row r="376" spans="5:13">
+    <row r="376" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E376" s="1"/>
       <c r="L376" s="1"/>
       <c r="M376" s="1"/>
     </row>
-    <row r="377" spans="5:13">
+    <row r="377" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E377" s="1"/>
       <c r="L377" s="1"/>
       <c r="M377" s="1"/>
     </row>
-    <row r="378" spans="5:13">
+    <row r="378" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E378" s="1"/>
       <c r="L378" s="1"/>
       <c r="M378" s="1"/>
     </row>
-    <row r="379" spans="5:13">
+    <row r="379" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E379" s="1"/>
       <c r="L379" s="1"/>
       <c r="M379" s="1"/>
     </row>
-    <row r="380" spans="5:13">
+    <row r="380" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E380" s="1"/>
       <c r="L380" s="1"/>
       <c r="M380" s="1"/>
     </row>
-    <row r="381" spans="5:13">
+    <row r="381" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E381" s="1"/>
       <c r="L381" s="1"/>
       <c r="M381" s="1"/>
     </row>
-    <row r="382" spans="5:13">
+    <row r="382" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E382" s="1"/>
       <c r="L382" s="1"/>
       <c r="M382" s="1"/>
     </row>
-    <row r="383" spans="5:13">
+    <row r="383" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E383" s="1"/>
       <c r="L383" s="1"/>
       <c r="M383" s="1"/>
     </row>
-    <row r="384" spans="5:13">
+    <row r="384" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E384" s="1"/>
       <c r="L384" s="1"/>
       <c r="M384" s="1"/>
     </row>
-    <row r="385" spans="5:13">
+    <row r="385" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E385" s="1"/>
       <c r="L385" s="1"/>
       <c r="M385" s="1"/>
     </row>
-    <row r="386" spans="5:13">
+    <row r="386" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E386" s="1"/>
       <c r="L386" s="1"/>
       <c r="M386" s="1"/>
     </row>
-    <row r="387" spans="5:13">
+    <row r="387" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E387" s="1"/>
       <c r="L387" s="1"/>
       <c r="M387" s="1"/>
     </row>
-    <row r="388" spans="5:13">
+    <row r="388" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E388" s="1"/>
       <c r="L388" s="1"/>
       <c r="M388" s="1"/>
     </row>
-    <row r="389" spans="5:13">
+    <row r="389" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E389" s="1"/>
       <c r="L389" s="1"/>
       <c r="M389" s="1"/>
     </row>
-    <row r="390" spans="5:13">
+    <row r="390" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E390" s="1"/>
       <c r="L390" s="1"/>
       <c r="M390" s="1"/>
     </row>
-    <row r="391" spans="5:13">
+    <row r="391" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E391" s="1"/>
       <c r="L391" s="1"/>
       <c r="M391" s="1"/>
     </row>
-    <row r="392" spans="5:13">
+    <row r="392" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E392" s="1"/>
       <c r="L392" s="1"/>
       <c r="M392" s="1"/>
     </row>
-    <row r="393" spans="5:13">
+    <row r="393" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E393" s="1"/>
       <c r="L393" s="1"/>
       <c r="M393" s="1"/>
     </row>
-    <row r="394" spans="5:13">
+    <row r="394" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E394" s="1"/>
       <c r="L394" s="1"/>
       <c r="M394" s="1"/>
     </row>
-    <row r="395" spans="5:13">
+    <row r="395" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E395" s="1"/>
       <c r="L395" s="1"/>
       <c r="M395" s="1"/>
     </row>
-    <row r="396" spans="5:13">
+    <row r="396" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E396" s="1"/>
       <c r="L396" s="1"/>
       <c r="M396" s="1"/>
     </row>
-    <row r="397" spans="5:13">
+    <row r="397" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E397" s="1"/>
       <c r="L397" s="1"/>
       <c r="M397" s="1"/>
     </row>
-    <row r="398" spans="5:13">
+    <row r="398" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E398" s="1"/>
       <c r="L398" s="1"/>
       <c r="M398" s="1"/>
     </row>
-    <row r="399" spans="5:13">
+    <row r="399" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E399" s="1"/>
       <c r="L399" s="1"/>
       <c r="M399" s="1"/>
     </row>
-    <row r="400" spans="5:13">
+    <row r="400" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E400" s="1"/>
       <c r="L400" s="1"/>
       <c r="M400" s="1"/>
     </row>
-    <row r="401" spans="5:13">
+    <row r="401" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E401" s="1"/>
       <c r="L401" s="1"/>
       <c r="M401" s="1"/>
     </row>
-    <row r="402" spans="5:13">
+    <row r="402" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E402" s="1"/>
       <c r="L402" s="1"/>
       <c r="M402" s="1"/>
     </row>
-    <row r="403" spans="5:13">
+    <row r="403" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E403" s="1"/>
       <c r="L403" s="1"/>
       <c r="M403" s="1"/>
     </row>
-    <row r="404" spans="5:13">
+    <row r="404" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E404" s="1"/>
       <c r="L404" s="1"/>
       <c r="M404" s="1"/>
     </row>
-    <row r="405" spans="5:13">
+    <row r="405" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E405" s="1"/>
       <c r="L405" s="1"/>
       <c r="M405" s="1"/>
     </row>
-    <row r="406" spans="5:13">
+    <row r="406" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E406" s="1"/>
       <c r="L406" s="1"/>
       <c r="M406" s="1"/>
     </row>
-    <row r="407" spans="5:13">
+    <row r="407" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E407" s="1"/>
       <c r="L407" s="1"/>
       <c r="M407" s="1"/>
     </row>
-    <row r="408" spans="5:13">
+    <row r="408" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E408" s="1"/>
       <c r="L408" s="1"/>
       <c r="M408" s="1"/>
     </row>
-    <row r="409" spans="5:13">
+    <row r="409" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E409" s="1"/>
       <c r="L409" s="1"/>
       <c r="M409" s="1"/>
     </row>
-    <row r="410" spans="5:13">
+    <row r="410" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E410" s="1"/>
       <c r="L410" s="1"/>
       <c r="M410" s="1"/>
     </row>
-    <row r="411" spans="5:13">
+    <row r="411" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E411" s="1"/>
       <c r="L411" s="1"/>
       <c r="M411" s="1"/>
     </row>
-    <row r="412" spans="5:13">
+    <row r="412" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E412" s="1"/>
       <c r="L412" s="1"/>
       <c r="M412" s="1"/>
     </row>
-    <row r="413" spans="5:13">
+    <row r="413" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E413" s="1"/>
       <c r="L413" s="1"/>
       <c r="M413" s="1"/>
     </row>
-    <row r="414" spans="5:13">
+    <row r="414" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E414" s="1"/>
       <c r="L414" s="1"/>
       <c r="M414" s="1"/>
     </row>
-    <row r="415" spans="5:13">
+    <row r="415" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E415" s="1"/>
       <c r="L415" s="1"/>
       <c r="M415" s="1"/>
     </row>
-    <row r="416" spans="5:13">
+    <row r="416" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E416" s="1"/>
       <c r="L416" s="1"/>
       <c r="M416" s="1"/>
     </row>
-    <row r="417" spans="5:13">
+    <row r="417" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E417" s="1"/>
       <c r="L417" s="1"/>
       <c r="M417" s="1"/>
     </row>
-    <row r="418" spans="5:13">
+    <row r="418" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E418" s="1"/>
       <c r="L418" s="1"/>
       <c r="M418" s="1"/>
     </row>
-    <row r="419" spans="5:13">
+    <row r="419" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E419" s="1"/>
       <c r="L419" s="1"/>
       <c r="M419" s="1"/>
     </row>
-    <row r="420" spans="5:13">
+    <row r="420" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E420" s="1"/>
       <c r="L420" s="1"/>
       <c r="M420" s="1"/>
     </row>
-    <row r="421" spans="5:13">
+    <row r="421" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E421" s="1"/>
       <c r="L421" s="1"/>
       <c r="M421" s="1"/>
     </row>
-    <row r="422" spans="5:13">
+    <row r="422" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E422" s="1"/>
       <c r="L422" s="1"/>
       <c r="M422" s="1"/>
     </row>
-    <row r="423" spans="5:13">
+    <row r="423" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E423" s="1"/>
       <c r="L423" s="1"/>
       <c r="M423" s="1"/>
     </row>
-    <row r="424" spans="5:13">
+    <row r="424" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E424" s="1"/>
       <c r="L424" s="1"/>
       <c r="M424" s="1"/>
     </row>
-    <row r="425" spans="5:13">
+    <row r="425" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E425" s="1"/>
       <c r="L425" s="1"/>
       <c r="M425" s="1"/>
     </row>
-    <row r="426" spans="5:13">
+    <row r="426" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E426" s="1"/>
       <c r="L426" s="1"/>
       <c r="M426" s="1"/>
     </row>
-    <row r="427" spans="5:13">
+    <row r="427" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E427" s="1"/>
       <c r="L427" s="1"/>
       <c r="M427" s="1"/>
     </row>
-    <row r="428" spans="5:13">
+    <row r="428" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E428" s="1"/>
       <c r="L428" s="1"/>
       <c r="M428" s="1"/>
     </row>
-    <row r="429" spans="5:13">
+    <row r="429" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E429" s="1"/>
       <c r="L429" s="1"/>
       <c r="M429" s="1"/>
     </row>
-    <row r="430" spans="5:13">
+    <row r="430" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E430" s="1"/>
       <c r="L430" s="1"/>
       <c r="M430" s="1"/>
     </row>
-    <row r="431" spans="5:13">
+    <row r="431" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E431" s="1"/>
       <c r="L431" s="1"/>
       <c r="M431" s="1"/>
     </row>
-    <row r="432" spans="5:13">
+    <row r="432" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E432" s="1"/>
       <c r="L432" s="1"/>
       <c r="M432" s="1"/>
     </row>
-    <row r="433" spans="5:13">
+    <row r="433" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E433" s="1"/>
       <c r="L433" s="1"/>
       <c r="M433" s="1"/>
     </row>
-    <row r="434" spans="5:13">
+    <row r="434" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E434" s="1"/>
       <c r="L434" s="1"/>
       <c r="M434" s="1"/>
     </row>
-    <row r="435" spans="5:13">
+    <row r="435" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E435" s="1"/>
       <c r="L435" s="1"/>
       <c r="M435" s="1"/>
     </row>
-    <row r="436" spans="5:13">
+    <row r="436" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E436" s="1"/>
       <c r="L436" s="1"/>
       <c r="M436" s="1"/>
     </row>
-    <row r="437" spans="5:13">
+    <row r="437" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E437" s="1"/>
       <c r="L437" s="1"/>
       <c r="M437" s="1"/>
     </row>
-    <row r="438" spans="5:13">
+    <row r="438" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E438" s="1"/>
       <c r="L438" s="1"/>
       <c r="M438" s="1"/>
     </row>
-    <row r="439" spans="5:13">
+    <row r="439" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E439" s="1"/>
       <c r="L439" s="1"/>
       <c r="M439" s="1"/>
     </row>
-    <row r="440" spans="5:13">
+    <row r="440" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E440" s="1"/>
       <c r="L440" s="1"/>
       <c r="M440" s="1"/>
     </row>
-    <row r="441" spans="5:13">
+    <row r="441" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E441" s="1"/>
       <c r="L441" s="1"/>
       <c r="M441" s="1"/>
     </row>
-    <row r="442" spans="5:13">
+    <row r="442" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E442" s="1"/>
       <c r="L442" s="1"/>
       <c r="M442" s="1"/>
     </row>
-    <row r="443" spans="5:13">
+    <row r="443" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E443" s="1"/>
       <c r="L443" s="1"/>
       <c r="M443" s="1"/>
     </row>
-    <row r="444" spans="5:13">
+    <row r="444" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E444" s="1"/>
       <c r="L444" s="1"/>
       <c r="M444" s="1"/>
     </row>
-    <row r="445" spans="5:13">
+    <row r="445" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E445" s="1"/>
       <c r="L445" s="1"/>
       <c r="M445" s="1"/>
     </row>
-    <row r="446" spans="5:13">
+    <row r="446" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E446" s="1"/>
       <c r="L446" s="1"/>
       <c r="M446" s="1"/>
     </row>
-    <row r="447" spans="5:13">
+    <row r="447" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E447" s="1"/>
       <c r="L447" s="1"/>
       <c r="M447" s="1"/>
     </row>
-    <row r="448" spans="5:13">
+    <row r="448" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E448" s="1"/>
       <c r="L448" s="1"/>
       <c r="M448" s="1"/>
     </row>
-    <row r="449" spans="5:13">
+    <row r="449" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E449" s="1"/>
       <c r="L449" s="1"/>
       <c r="M449" s="1"/>
     </row>
-    <row r="450" spans="5:13">
+    <row r="450" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E450" s="1"/>
       <c r="L450" s="1"/>
       <c r="M450" s="1"/>
     </row>
-    <row r="451" spans="5:13">
+    <row r="451" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E451" s="1"/>
       <c r="L451" s="1"/>
       <c r="M451" s="1"/>
     </row>
-    <row r="452" spans="5:13">
+    <row r="452" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E452" s="1"/>
       <c r="L452" s="1"/>
       <c r="M452" s="1"/>
     </row>
-    <row r="453" spans="5:13">
+    <row r="453" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E453" s="1"/>
       <c r="L453" s="1"/>
       <c r="M453" s="1"/>
     </row>
-    <row r="454" spans="5:13">
+    <row r="454" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E454" s="1"/>
       <c r="L454" s="1"/>
       <c r="M454" s="1"/>
     </row>
-    <row r="455" spans="5:13">
+    <row r="455" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E455" s="1"/>
       <c r="L455" s="1"/>
       <c r="M455" s="1"/>
     </row>
-    <row r="456" spans="5:13">
+    <row r="456" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E456" s="1"/>
       <c r="L456" s="1"/>
       <c r="M456" s="1"/>
     </row>
-    <row r="457" spans="5:13">
+    <row r="457" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E457" s="1"/>
       <c r="L457" s="1"/>
       <c r="M457" s="1"/>
     </row>
-    <row r="458" spans="5:13">
+    <row r="458" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E458" s="1"/>
       <c r="L458" s="1"/>
       <c r="M458" s="1"/>
     </row>
-    <row r="459" spans="5:13">
+    <row r="459" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E459" s="1"/>
       <c r="L459" s="1"/>
       <c r="M459" s="1"/>
     </row>
-    <row r="460" spans="5:13">
+    <row r="460" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E460" s="1"/>
       <c r="L460" s="1"/>
       <c r="M460" s="1"/>
     </row>
-    <row r="461" spans="5:13">
+    <row r="461" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E461" s="1"/>
       <c r="L461" s="1"/>
       <c r="M461" s="1"/>
     </row>
-    <row r="462" spans="5:13">
+    <row r="462" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E462" s="1"/>
       <c r="L462" s="1"/>
       <c r="M462" s="1"/>
     </row>
-    <row r="463" spans="5:13">
+    <row r="463" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E463" s="1"/>
       <c r="L463" s="1"/>
       <c r="M463" s="1"/>
     </row>
-    <row r="464" spans="5:13">
+    <row r="464" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E464" s="1"/>
       <c r="L464" s="1"/>
       <c r="M464" s="1"/>
     </row>
-    <row r="465" spans="5:13">
+    <row r="465" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E465" s="1"/>
       <c r="L465" s="1"/>
       <c r="M465" s="1"/>
     </row>
-    <row r="466" spans="5:13">
+    <row r="466" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E466" s="1"/>
       <c r="L466" s="1"/>
       <c r="M466" s="1"/>
     </row>
-    <row r="467" spans="5:13">
+    <row r="467" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E467" s="1"/>
       <c r="L467" s="1"/>
       <c r="M467" s="1"/>
     </row>
-    <row r="468" spans="5:13">
+    <row r="468" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E468" s="1"/>
       <c r="L468" s="1"/>
       <c r="M468" s="1"/>
     </row>
-    <row r="469" spans="5:13">
+    <row r="469" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E469" s="1"/>
       <c r="L469" s="1"/>
       <c r="M469" s="1"/>
     </row>
-    <row r="470" spans="5:13">
+    <row r="470" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E470" s="1"/>
       <c r="L470" s="1"/>
       <c r="M470" s="1"/>
     </row>
-    <row r="471" spans="5:13">
+    <row r="471" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E471" s="1"/>
       <c r="L471" s="1"/>
       <c r="M471" s="1"/>
     </row>
-    <row r="472" spans="5:13">
+    <row r="472" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E472" s="1"/>
       <c r="L472" s="1"/>
       <c r="M472" s="1"/>
     </row>
-    <row r="473" spans="5:13">
+    <row r="473" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E473" s="1"/>
       <c r="L473" s="1"/>
       <c r="M473" s="1"/>
     </row>
-    <row r="474" spans="5:13">
+    <row r="474" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E474" s="1"/>
       <c r="L474" s="1"/>
       <c r="M474" s="1"/>
     </row>
-    <row r="475" spans="5:13">
+    <row r="475" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E475" s="1"/>
       <c r="L475" s="1"/>
       <c r="M475" s="1"/>
     </row>
-    <row r="476" spans="5:13">
+    <row r="476" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E476" s="1"/>
       <c r="L476" s="1"/>
       <c r="M476" s="1"/>
     </row>
-    <row r="477" spans="5:13">
+    <row r="477" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E477" s="1"/>
       <c r="L477" s="1"/>
       <c r="M477" s="1"/>
     </row>
-    <row r="478" spans="5:13">
+    <row r="478" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E478" s="1"/>
       <c r="L478" s="1"/>
       <c r="M478" s="1"/>
     </row>
-    <row r="479" spans="5:13">
+    <row r="479" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E479" s="1"/>
       <c r="L479" s="1"/>
       <c r="M479" s="1"/>
     </row>
-    <row r="480" spans="5:13">
+    <row r="480" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E480" s="1"/>
       <c r="L480" s="1"/>
       <c r="M480" s="1"/>
     </row>
-    <row r="481" spans="5:13">
+    <row r="481" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E481" s="1"/>
       <c r="L481" s="1"/>
       <c r="M481" s="1"/>
     </row>
-    <row r="482" spans="5:13">
+    <row r="482" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E482" s="1"/>
       <c r="L482" s="1"/>
       <c r="M482" s="1"/>
     </row>
-    <row r="483" spans="5:13">
+    <row r="483" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E483" s="1"/>
       <c r="L483" s="1"/>
       <c r="M483" s="1"/>
     </row>
-    <row r="484" spans="5:13">
+    <row r="484" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E484" s="1"/>
       <c r="L484" s="1"/>
       <c r="M484" s="1"/>
     </row>
-    <row r="485" spans="5:13">
+    <row r="485" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E485" s="1"/>
       <c r="L485" s="1"/>
       <c r="M485" s="1"/>
+    </row>
+    <row r="486" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E486" s="1"/>
+      <c r="L486" s="1"/>
+      <c r="M486" s="1"/>
+    </row>
+    <row r="487" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E487" s="1"/>
+      <c r="L487" s="1"/>
+      <c r="M487" s="1"/>
+    </row>
+    <row r="488" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E488" s="1"/>
+      <c r="L488" s="1"/>
+      <c r="M488" s="1"/>
+    </row>
+    <row r="489" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E489" s="1"/>
+      <c r="L489" s="1"/>
+      <c r="M489" s="1"/>
+    </row>
+    <row r="490" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E490" s="1"/>
+      <c r="L490" s="1"/>
+      <c r="M490" s="1"/>
+    </row>
+    <row r="491" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E491" s="1"/>
+      <c r="L491" s="1"/>
+      <c r="M491" s="1"/>
+    </row>
+    <row r="492" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E492" s="1"/>
+      <c r="L492" s="1"/>
+      <c r="M492" s="1"/>
+    </row>
+    <row r="493" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E493" s="1"/>
+      <c r="L493" s="1"/>
+      <c r="M493" s="1"/>
+    </row>
+    <row r="494" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E494" s="1"/>
+      <c r="L494" s="1"/>
+      <c r="M494" s="1"/>
+    </row>
+    <row r="495" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E495" s="1"/>
+      <c r="L495" s="1"/>
+      <c r="M495" s="1"/>
+    </row>
+    <row r="496" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E496" s="1"/>
+      <c r="L496" s="1"/>
+      <c r="M496" s="1"/>
+    </row>
+    <row r="497" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E497" s="1"/>
+      <c r="L497" s="1"/>
+      <c r="M497" s="1"/>
+    </row>
+    <row r="498" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E498" s="1"/>
+      <c r="L498" s="1"/>
+      <c r="M498" s="1"/>
+    </row>
+    <row r="499" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E499" s="1"/>
+      <c r="L499" s="1"/>
+      <c r="M499" s="1"/>
+    </row>
+    <row r="500" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E500" s="1"/>
+      <c r="L500" s="1"/>
+      <c r="M500" s="1"/>
+    </row>
+    <row r="501" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E501" s="1"/>
+      <c r="L501" s="1"/>
+      <c r="M501" s="1"/>
+    </row>
+    <row r="502" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E502" s="1"/>
+      <c r="L502" s="1"/>
+      <c r="M502" s="1"/>
+    </row>
+    <row r="503" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E503" s="1"/>
+      <c r="L503" s="1"/>
+      <c r="M503" s="1"/>
+    </row>
+    <row r="504" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E504" s="1"/>
+      <c r="L504" s="1"/>
+      <c r="M504" s="1"/>
+    </row>
+    <row r="505" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E505" s="1"/>
+      <c r="L505" s="1"/>
+      <c r="M505" s="1"/>
+    </row>
+    <row r="506" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E506" s="1"/>
+      <c r="L506" s="1"/>
+      <c r="M506" s="1"/>
+    </row>
+    <row r="507" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E507" s="1"/>
+      <c r="L507" s="1"/>
+      <c r="M507" s="1"/>
+    </row>
+    <row r="508" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E508" s="1"/>
+      <c r="L508" s="1"/>
+      <c r="M508" s="1"/>
+    </row>
+    <row r="509" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E509" s="1"/>
+      <c r="L509" s="1"/>
+      <c r="M509" s="1"/>
+    </row>
+    <row r="510" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E510" s="1"/>
+      <c r="L510" s="1"/>
+      <c r="M510" s="1"/>
+    </row>
+    <row r="511" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E511" s="1"/>
+      <c r="L511" s="1"/>
+      <c r="M511" s="1"/>
+    </row>
+    <row r="512" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E512" s="1"/>
+      <c r="L512" s="1"/>
+      <c r="M512" s="1"/>
+    </row>
+    <row r="513" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E513" s="1"/>
+      <c r="L513" s="1"/>
+      <c r="M513" s="1"/>
+    </row>
+    <row r="514" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E514" s="1"/>
+      <c r="L514" s="1"/>
+      <c r="M514" s="1"/>
+    </row>
+    <row r="515" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E515" s="1"/>
+      <c r="L515" s="1"/>
+      <c r="M515" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>